<commit_message>
Simple Flow: regenerate Excel + TestRail import; add Open Questions for Milos
Rebuild SimpleFlow_V1_TestCases.xlsx/.csv and the TestRail import (159 cases;
0 VIU / 0 feature-flag / leaf sections / header-matched). Open Questions tab
now marks the 3 SV-8183-resolved items RESOLVED and keeps 11 open. Add a clean
standalone OpenQuestions-for-Milos.md/.xlsx (11 questions) via
gen_milos_questions.py, and update RESUME-STRATEGY / PROJECT-STATUS memory.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_V1_TestCases.xlsx
+++ b/build/simple-flow/SimpleFlow_V1_TestCases.xlsx
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -197,8 +197,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -580,7 +586,7 @@
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Simple Flow V1 (Simple Mode) - Manual Test Cases
-This workbook contains 156 manual test cases covering the ShopView "Simple Mode - Streamlined Work Order Completion &amp; Receiving" feature (Epic SV-7301): the Work Order settings page; the four settings-driven completion flows (No-PO/skip, PO+Optional invoice, PO+Required invoice, and Review-ON); the tech-story and line-approval gates; core-part resolution; vendorless / Vendor-Missing part handling; PO multi-select, Bulk Receive, apply-invoice, part-number fix, the WO-PO Receive button, Accept Delivery and assign-vendor / merge; the Waiting-on-Parts column; UX refinements; permissions; validation / edge cases; and QuickBooks / inventory integrity.
+This workbook contains 159 manual test cases covering the ShopView "Simple Mode - Streamlined Work Order Completion &amp; Receiving" feature (Epic SV-7301): the Work Order settings page; the four settings-driven completion flows (No-PO/skip, PO+Optional invoice, PO+Required invoice, and Review-ON); the tech-story and line-approval gates; core-part resolution; vendorless / Vendor-Missing part handling; PO multi-select, Bulk Receive, apply-invoice, part-number fix, the WO-PO Receive button, Accept Delivery and assign-vendor / merge; the Waiting-on-Parts column; UX refinements; permissions; validation / edge cases; and QuickBooks / inventory integrity.
 Authored from the COMPLETE spec (build/simple-flow/requirements.md, 17 stories) plus the design mockups / dev handoffs (design-notes.md) and the live VIU findings (viu-findings.md).
 VIU (Verify-in-UI on QA env sv7301) is PARTIAL because the feature is still under development. Each case carries a VIU Status: VIU-Verified (tested live and passed - screenshot cited in Notes), VIU-Pending (not yet verifiable - either a not-built story or a cookie/role-dependent check), or Open-Question (the expected result depends on an unresolved decision or a VIU deviation - see the Open Questions tab).
 NOT-BUILT stories (all cases VIU-Pending until dev completes): Story 7 (PO multi-select), Story 8 (Bulk Receive page), Story 9 (apply-invoice), Story 14 (Waiting-on-Parts column).
@@ -804,7 +810,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
@@ -834,7 +840,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29">
@@ -873,7 +879,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33">
@@ -903,7 +909,7 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="37">
@@ -942,7 +948,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41">
@@ -952,7 +958,7 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
@@ -962,7 +968,7 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="44" ht="160" customHeight="1">
@@ -971,8 +977,8 @@
           <t>Legend &amp; notes:
 - VIU-Verified = tested live on QA env sv7301 and passed (screenshot cited in the case Notes).
 - VIU-Pending = still needs live verification: either a NOT-BUILT story (7 Bulk multi-select, 8 Bulk Receive page, 9 apply-invoice, 14 Waiting-on-Parts) or a cookie/role-dependent check (non-admin role-gating negatives; full parts-receive + core round-trips; line-approval final block). See the 'VIU pending' tab.
-- Open-Question = the EXPECTED result depends on an unresolved decision or a VIU deviation/bug. See the 'Open Questions' tab (14 items, including the 4 live VIU deviations).
-- No permissions/role matrix exists yet: role-gating cases are authored but their expected results are marked TBD - do not assume role outcomes.</t>
+- Open-Question = the EXPECTED result depends on an unresolved decision or a live build deviation. See the 'Open Questions' tab (14 items: 3 RESOLVED by SV-8183, 11 still open pending Milos).
+- Permissions are now DEFINED by SV-8183: Simple Flow reuses existing Custom Roles atoms (no new atom) plus the NET-NEW reviewer!=completer rule. See requirements §9 for the action-&gt;atom map and per-role matrix; role-gating negatives still need live verification.</t>
         </is>
       </c>
     </row>
@@ -991,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M157"/>
+  <dimension ref="A1:M160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1832,31 +1838,32 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD). A non-admin (e.g. Advisor/Tech) credential is required.</t>
+          <t>App Settings permission (system defaults: Admin, Service Manager, Office). A role WITHOUT App Settings (e.g. Service Advisor / Technician) is required for this negative.</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t>1. A non-admin user account exists for this org.
-2. You can sign in as that non-admin user.</t>
+          <t>1. A user without the App Settings permission (e.g. Service Advisor or Technician) exists for this org.
+2. You can sign in as that user.</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
-          <t>1. Sign in as the non-admin user.
+          <t>1. Sign in as the user without App Settings.
 2. Attempt to open /administration/settings → Work Orders tab.
-3. Attempt to change and save a Work Order setting.</t>
+3. Attempt to change and save a Work Order setting, including a direct API save.</t>
         </is>
       </c>
       <c r="J12" s="17" t="inlineStr">
         <is>
-          <t>1. The non-admin cannot reach the Work Order settings, OR the settings are read-only for them.
-2. The non-admin cannot save changes to Work Order settings.</t>
+          <t>1. A role without the App Settings permission cannot reach the Work Order settings, or sees them read-only.
+2. That role cannot save changes to Work Order settings.
+3. The backend rejects a Work Order settings save attempted by a role that lacks App Settings.</t>
         </is>
       </c>
       <c r="K12" s="17" t="inlineStr">
         <is>
-          <t>requirements S1 AC</t>
+          <t>requirements S1 AC / §9 (App Settings gate)</t>
         </is>
       </c>
       <c r="L12" s="24" t="inlineStr">
@@ -1866,7 +1873,7 @@
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>BLOCKED in VIU: quick-login {key:'tech'} returned 403 in this env; only the admin session works. Needs a real non-admin credential. Expected also depends on the (TBD) permissions matrix.</t>
+          <t>Defined by SV-8183: the Work Order settings inherit the settingsApp route guard (no new atom); editable only by roles with App Settings ON (defaults Admin, Service Manager, Office). Role-gating negatives not yet verified live (only the admin session works on sv7301; tech key = 403).</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5137,7 @@
       </c>
       <c r="G58" s="17" t="inlineStr">
         <is>
-          <t>Work Order edit access (add parts).</t>
+          <t>WO Lines: Create &amp; Edit + See Financial Data (the sell price is mandatory and has no catalog source).</t>
         </is>
       </c>
       <c r="H58" s="17" t="inlineStr">
@@ -5151,12 +5158,13 @@
         <is>
           <t>1. The part saves successfully.
 2. The part appears on the line with its description, quantity and sell price.
-3. It is treated as a vendorless part downstream.</t>
+3. It is treated as a vendorless part downstream.
+4. Adding a vendorless / no-part-number part requires WO Lines: Create &amp; Edit and See Financial Data, because the sell price is mandatory and has no catalog source.</t>
         </is>
       </c>
       <c r="K58" s="17" t="inlineStr">
         <is>
-          <t>requirements S5-R1</t>
+          <t>requirements S5-R1 / §9 (See Financial Data gate)</t>
         </is>
       </c>
       <c r="L58" s="24" t="inlineStr">
@@ -5166,7 +5174,7 @@
       </c>
       <c r="M58" s="17" t="inlineStr">
         <is>
-          <t>Not driven in VIU (part-add flow not exercised). Needs live verification.</t>
+          <t>SV-8183 Decision 4 adds a financial gate: vendorless / no-PN add requires See Financial Data (mandatory sell). Not driven live (part-add flow not exercised).</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5211,7 @@
       </c>
       <c r="G59" s="21" t="inlineStr">
         <is>
-          <t>Work Order edit access (add parts).</t>
+          <t>WO Lines: Create &amp; Edit + See Financial Data. A role lacking See Financial Data (e.g. Technician) is used for the permission negative.</t>
         </is>
       </c>
       <c r="H59" s="21" t="inlineStr">
@@ -5216,19 +5224,21 @@
         <is>
           <t>1. Leave the description empty and try to save.
 2. Fill description, leave quantity empty and try to save.
-3. Fill quantity, leave sell price empty and try to save.</t>
+3. Fill quantity, leave sell price empty and try to save.
+4. As a role without See Financial Data (e.g. Technician), attempt to add a vendorless / no-part-number part.</t>
         </is>
       </c>
       <c r="J59" s="21" t="inlineStr">
         <is>
           <t>1. Saving is blocked when the description is empty.
 2. Saving is blocked when the quantity is empty.
-3. Saving is blocked when the sell price is empty.</t>
+3. Saving is blocked when the sell price is empty.
+4. A user without See Financial Data (for example a Technician) cannot add a vendorless / no-part-number part, because they cannot enter the mandatory sell price.</t>
         </is>
       </c>
       <c r="K59" s="21" t="inlineStr">
         <is>
-          <t>requirements S5 AC</t>
+          <t>requirements S5 AC / §9 (See Financial Data gate)</t>
         </is>
       </c>
       <c r="L59" s="24" t="inlineStr">
@@ -5238,7 +5248,7 @@
       </c>
       <c r="M59" s="21" t="inlineStr">
         <is>
-          <t>Not driven in VIU. Needs live verification of the exact rejection UX.</t>
+          <t>SV-8183 Decision 4: vendorless / no-PN add requires See Financial Data. Field validation and the permission negative not yet verified live.</t>
         </is>
       </c>
     </row>
@@ -7974,31 +7984,31 @@
       </c>
       <c r="G98" s="17" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD). Office/readonly credential required.</t>
+          <t>Order Parts permission (absent for Office / read-only roles).</t>
         </is>
       </c>
       <c r="H98" s="17" t="inlineStr">
         <is>
-          <t>1. An office / readonly user credential exists.
+          <t>1. An Office / read-only user credential (no Order Parts) exists.
 2. A fulfilled PO and an unfulfilled PO exist.</t>
         </is>
       </c>
       <c r="I98" s="17" t="inlineStr">
         <is>
-          <t>1. Sign in as an office/readonly user and open the PO list.
+          <t>1. Sign in as an Office / read-only user and open the PO list.
 2. Confirm the Receive action is hidden for them.
 3. As an authorized user, confirm the Receive action is hidden on a fulfilled PO.</t>
         </is>
       </c>
       <c r="J98" s="17" t="inlineStr">
         <is>
-          <t>1. EXPECTED PER SPEC: office/readonly users do not see the Receive action (final expected depends on the permissions matrix — TBD).
+          <t>1. The Receive action requires the Order Parts permission; Office and read-only users (no Order Parts) do not see Receive on the PO list or detail.
 2. Fulfilled POs do not show the Receive action.</t>
         </is>
       </c>
       <c r="K98" s="17" t="inlineStr">
         <is>
-          <t>requirements S11-R3</t>
+          <t>requirements S11-R3 / §9 (Order Parts gate)</t>
         </is>
       </c>
       <c r="L98" s="24" t="inlineStr">
@@ -8008,7 +8018,7 @@
       </c>
       <c r="M98" s="17" t="inlineStr">
         <is>
-          <t>Role-gating negative not verifiable in VIU (no non-admin session; tech key = 403). Expected depends on the (TBD) permissions matrix. Fulfilled-PO hiding needs live verification.</t>
+          <t>SV-8183 resolves 'office/readonly' to concrete atoms: Receive-on-WO is FE-gated by Order Parts; Office (WO View-only / Vendor &amp; Order View-only) lacks it. Role-gating negative not yet verified live. Fulfilled-PO hiding also needs live verification.</t>
         </is>
       </c>
     </row>
@@ -9589,7 +9599,7 @@
       </c>
       <c r="D121" s="21" t="inlineStr">
         <is>
-          <t>Verify Mark Reviewed is available only to manager/foreman and disabled for an advisor with 'Awaiting review'</t>
+          <t>Verify Mark Reviewed is gated by the Review Work Orders permission and disabled for a role without it</t>
         </is>
       </c>
       <c r="E121" s="22" t="inlineStr">
@@ -9604,31 +9614,32 @@
       </c>
       <c r="G121" s="21" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD). Reviewer (manager/foreman) and advisor credentials required.</t>
+          <t>Review Work Orders permission + reviewer must not be the completer.</t>
         </is>
       </c>
       <c r="H121" s="21" t="inlineStr">
         <is>
-          <t>1. Manager/foreman and advisor credentials exist.
-2. A work order is in Review state.</t>
+          <t>1. A role with Review Work Orders and a role without it both exist.
+2. A work order is in Review state, sent to review by a known user.</t>
         </is>
       </c>
       <c r="I121" s="21" t="inlineStr">
         <is>
-          <t>1. Sign in as an advisor and open the work order in Review.
+          <t>1. Sign in as a role without Review Work Orders and open the work order in Review.
 2. Confirm Mark Reviewed is disabled with 'Awaiting review'.
-3. Sign in as a manager/foreman and confirm Mark Reviewed is available.</t>
+3. Sign in as a role with Review Work Orders (system defaults grant it broadly; it can be limited to manager/foreman via custom roles) and confirm Mark Reviewed is available.</t>
         </is>
       </c>
       <c r="J121" s="21" t="inlineStr">
         <is>
-          <t>1. EXPECTED PER SPEC: advisors see Mark Reviewed disabled with 'Awaiting review'.
-2. Managers/foremen can Mark Reviewed. (Final expected depends on the permissions matrix — TBD.)</t>
+          <t>1. A role without the Review Work Orders permission sees Mark Reviewed disabled with an 'Awaiting review' indicator.
+2. A role with the Review Work Orders permission can Mark Reviewed and sign off.
+3. The user who completed / sent the work order to review cannot Mark Reviewed even with the permission; a different qualified reviewer can.</t>
         </is>
       </c>
       <c r="K121" s="21" t="inlineStr">
         <is>
-          <t>requirements R7</t>
+          <t>requirements R7 / §9 (Review Work Orders + reviewer != completer)</t>
         </is>
       </c>
       <c r="L121" s="24" t="inlineStr">
@@ -9638,7 +9649,7 @@
       </c>
       <c r="M121" s="21" t="inlineStr">
         <is>
-          <t>Role-gating not testable in VIU (admin-only session; tech key = 403). Expected depends on the (TBD) permissions matrix and the open 'role-gating review: custom roles vs open for v1' question. See Open Questions.</t>
+          <t>Defined by SV-8183: Mark Reviewed = Review Work Orders atom (defaults broad, narrowable to manager/foreman) plus reviewer != completer. Role-gating negatives not yet verified live (admin-only session on sv7301).</t>
         </is>
       </c>
     </row>
@@ -10044,7 +10055,7 @@
       </c>
       <c r="J127" s="21" t="inlineStr">
         <is>
-          <t>1. PENDING DECISION: the Require Review default follows the agreed cohort rule (e.g. on for bigger/existing shops), with existing orgs preserved via backfill.</t>
+          <t>1. A brand-new org shows the Require Review setting in its default state, and existing orgs keep their current completion behavior (the setting is backfilled so their behavior does not change).</t>
         </is>
       </c>
       <c r="K127" s="21" t="inlineStr">
@@ -10325,7 +10336,7 @@
       </c>
       <c r="J131" s="21" t="inlineStr">
         <is>
-          <t>1. PENDING DESIGN: Close closes the modal only (no discard) and stays on the work order.
+          <t>1. Clicking Close closes the modal only, keeps any entered changes, and stays on the work order.
 2. Cancel closes the modal and returns to the previous screen.</t>
         </is>
       </c>
@@ -10378,29 +10389,32 @@
       </c>
       <c r="G132" s="17" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD). Non-admin credential required.</t>
+          <t>App Settings permission (system defaults: Admin, Service Manager, Office). A role without App Settings is used for the negative.</t>
         </is>
       </c>
       <c r="H132" s="17" t="inlineStr">
         <is>
-          <t>1. A non-admin user account exists.
-2. You can sign in as that user.</t>
+          <t>1. A role with the App Settings permission (e.g. Admin) and a role without it (e.g. Service Advisor or Technician) both exist.
+2. You can sign in as each.</t>
         </is>
       </c>
       <c r="I132" s="17" t="inlineStr">
         <is>
-          <t>1. Sign in as the non-admin user.
-2. Attempt to open and modify /administration/settings → Work Orders.</t>
+          <t>1. Sign in as a role with App Settings and open and modify /administration/settings → Work Orders.
+2. Sign in as a role without App Settings and attempt to open and modify the same page.
+3. As the role without App Settings, attempt to save a Work Order settings change directly (API), and note the response.</t>
         </is>
       </c>
       <c r="J132" s="17" t="inlineStr">
         <is>
-          <t>1. The non-admin cannot view or modify Work Order settings (final expected depends on the permissions matrix — TBD).</t>
+          <t>1. Only a role with the App Settings permission (system defaults Admin, Service Manager and Office) can view and modify the Work Order settings page.
+2. A role without App Settings cannot open or change the Work Order settings.
+3. The backend rejects a Work Order settings save attempted by a role that lacks App Settings.</t>
         </is>
       </c>
       <c r="K132" s="17" t="inlineStr">
         <is>
-          <t>requirements S1 AC</t>
+          <t>requirements S1 AC / §9 (App Settings gate)</t>
         </is>
       </c>
       <c r="L132" s="24" t="inlineStr">
@@ -10410,7 +10424,7 @@
       </c>
       <c r="M132" s="17" t="inlineStr">
         <is>
-          <t>BLOCKED in VIU (quick-login tech = 403; no non-admin session). Needs a real non-admin credential. Hypothesis to verify: backend may only enforce resource-level View/Edit while these are FE display gates (Custom Roles finding). See Open Questions.</t>
+          <t>Permission defined by SV-8183: the Work Order settings inherit the existing settingsApp route guard (no new atom); editable by any role with App Settings ON (defaults Admin, Service Manager, Office). Note Office can edit settings but cannot operate the flow. Role-gating negatives not yet verified live (only the admin session works on sv7301).</t>
         </is>
       </c>
     </row>
@@ -10447,7 +10461,7 @@
       </c>
       <c r="G133" s="21" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD). Multiple role credentials required.</t>
+          <t>Work Orders: Create &amp; Edit + WO Lines: Create &amp; Edit + Full View (to approve lines).</t>
         </is>
       </c>
       <c r="H133" s="21" t="inlineStr">
@@ -10464,22 +10478,24 @@
       </c>
       <c r="J133" s="21" t="inlineStr">
         <is>
-          <t>1. PENDING MATRIX: expected depends on the permissions matrix (TBD). Do not assume specific role outcomes.</t>
+          <t>1. Roles with Work Orders: Create &amp; Edit plus WO Lines: Create &amp; Edit and Full View (needed to approve all lines) can complete a work order: Admin, Service Manager, Senior SA, Service Advisor, Foreman and Parts Manager.
+2. Technician and Parts Tech cannot complete (Technician cannot approve lines in Tech View and/or lacks Work Orders: Create &amp; Edit; Parts Tech is a receiver, not a completer).
+3. Office, Sales Rep and Time Clock cannot complete a work order.</t>
         </is>
       </c>
       <c r="K133" s="21" t="inlineStr">
         <is>
-          <t>requirements §8 open questions</t>
-        </is>
-      </c>
-      <c r="L133" s="18" t="inlineStr">
-        <is>
-          <t>Open-Question</t>
+          <t>requirements §9 (Complete WO gate + per-role matrix)</t>
+        </is>
+      </c>
+      <c r="L133" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="M133" s="21" t="inlineStr">
         <is>
-          <t>No permissions/role matrix supplied. Author only; expected depends on the matrix (TBD). See Open Questions.</t>
+          <t>Expected defined by the SV-8183 role matrix. Role-gating negatives not yet verified live (only the admin session works on sv7301).</t>
         </is>
       </c>
     </row>
@@ -10516,7 +10532,7 @@
       </c>
       <c r="G134" s="17" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD).</t>
+          <t>Vendor &amp; Order Mgmt: Create &amp; Edit + See Financial Data.</t>
         </is>
       </c>
       <c r="H134" s="17" t="inlineStr">
@@ -10533,22 +10549,24 @@
       </c>
       <c r="J134" s="17" t="inlineStr">
         <is>
-          <t>1. PENDING MATRIX: expected depends on the permissions matrix (TBD).</t>
+          <t>1. Roles with Vendor &amp; Order Mgmt: Create &amp; Edit plus See Financial Data can reach and use Bulk Receive: Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager and Parts Tech.
+2. Office (Vendor &amp; Order Mgmt: View only) can open the Bulk Receive page but cannot receive.
+3. Sales Rep and Time Clock cannot reach Bulk Receive.</t>
         </is>
       </c>
       <c r="K134" s="17" t="inlineStr">
         <is>
-          <t>requirements §8 open questions</t>
-        </is>
-      </c>
-      <c r="L134" s="18" t="inlineStr">
-        <is>
-          <t>Open-Question</t>
+          <t>requirements §9 (Bulk Receive gate + per-role matrix)</t>
+        </is>
+      </c>
+      <c r="L134" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="M134" s="17" t="inlineStr">
         <is>
-          <t>No matrix supplied; also Bulk Receive is not yet built. See Open Questions.</t>
+          <t>Expected defined by the SV-8183 role matrix (Bulk Receive = Vendor &amp; Order Mgmt C&amp;E + See Financial Data; Office is view-only). Bulk Receive is also not yet built. Role-gating negatives not yet verified live.</t>
         </is>
       </c>
     </row>
@@ -10585,13 +10603,13 @@
       </c>
       <c r="G135" s="21" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD). Manager/foreman + other role credentials required.</t>
+          <t>Review Work Orders permission + reviewer must not be the completer.</t>
         </is>
       </c>
       <c r="H135" s="21" t="inlineStr">
         <is>
-          <t>1. Credentials for manager/foreman and other roles exist.
-2. A work order in Review state exists.</t>
+          <t>1. Credentials for roles with and without Review Work Orders exist.
+2. A work order in Review state exists, sent to review by a known user.</t>
         </is>
       </c>
       <c r="I135" s="21" t="inlineStr">
@@ -10602,22 +10620,24 @@
       </c>
       <c r="J135" s="21" t="inlineStr">
         <is>
-          <t>1. PENDING MATRIX: spec says manager/foreman only, but role-gating (custom roles vs open for v1) is UNRESOLVED. Expected depends on the matrix (TBD).</t>
+          <t>1. Mark Reviewed (review sign-off) requires the Review Work Orders permission; system defaults grant it broadly, and it can be narrowed to manager/foreman via custom roles.
+2. A role without Review Work Orders sees Mark Reviewed disabled with an 'Awaiting review' indicator.
+3. The user who completed / sent the work order to review cannot Mark Reviewed it; a different user who holds Review Work Orders can sign off.</t>
         </is>
       </c>
       <c r="K135" s="21" t="inlineStr">
         <is>
-          <t>requirements R7 / §8</t>
-        </is>
-      </c>
-      <c r="L135" s="18" t="inlineStr">
-        <is>
-          <t>Open-Question</t>
+          <t>requirements R7 / §9 (Review Work Orders + reviewer != completer)</t>
+        </is>
+      </c>
+      <c r="L135" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="M135" s="21" t="inlineStr">
         <is>
-          <t>Role-gating for review is an explicit open question. See Open Questions.</t>
+          <t>Defined by SV-8183: Mark Reviewed = Review Work Orders atom (not open-to-all) PLUS the NET-NEW reviewer != completer hard rule. Role-gating negatives not yet verified live.</t>
         </is>
       </c>
     </row>
@@ -10654,30 +10674,31 @@
       </c>
       <c r="G136" s="17" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD). Office/readonly credential required.</t>
+          <t>Order Parts permission (absent for Office / read-only roles).</t>
         </is>
       </c>
       <c r="H136" s="17" t="inlineStr">
         <is>
-          <t>1. An office/readonly credential exists.
-2. A WO-originated PO exists.</t>
+          <t>1. An Office / read-only credential (no Order Parts) exists.
+2. A WO-originated PO exists, plus a fulfilled PO.</t>
         </is>
       </c>
       <c r="I136" s="17" t="inlineStr">
         <is>
-          <t>1. Sign in as an office/readonly user.
+          <t>1. Sign in as an Office / read-only user.
 2. Open the PO list and detail.
-3. Confirm the Receive action is not shown.</t>
+3. Confirm the Receive action is not shown, and confirm it is also absent on a fulfilled PO.</t>
         </is>
       </c>
       <c r="J136" s="17" t="inlineStr">
         <is>
-          <t>1. EXPECTED PER SPEC: office/readonly users do not see the Receive action (final expected depends on the permissions matrix — TBD).</t>
+          <t>1. The Receive action requires the Order Parts permission; Office and read-only users (no Order Parts) do not see Receive on the PO list or PO detail.
+2. Receive is also hidden for fulfilled (already-received) POs.</t>
         </is>
       </c>
       <c r="K136" s="17" t="inlineStr">
         <is>
-          <t>requirements S11-R3</t>
+          <t>requirements S11-R3 / §9 (Order Parts gate)</t>
         </is>
       </c>
       <c r="L136" s="24" t="inlineStr">
@@ -10687,7 +10708,7 @@
       </c>
       <c r="M136" s="17" t="inlineStr">
         <is>
-          <t>Not verifiable in VIU (no non-admin session). Needs an office/readonly credential. See Open Questions.</t>
+          <t>SV-8183 resolves 'office/readonly' to concrete atoms: Receive-on-WO is FE-gated by Order Parts; Office (WO View-only / Vendor &amp; Order View-only) lacks it. Role-gating negatives not yet verified live.</t>
         </is>
       </c>
     </row>
@@ -10709,7 +10730,7 @@
       </c>
       <c r="D137" s="21" t="inlineStr">
         <is>
-          <t>Verify whether the backend enforces the Simple-Flow settings or they are front-end display gates only</t>
+          <t>Verify the backend enforces the Simple-Flow settings and permission atoms (not front-end only)</t>
         </is>
       </c>
       <c r="E137" s="23" t="inlineStr">
@@ -10735,28 +10756,31 @@
       </c>
       <c r="I137" s="21" t="inlineStr">
         <is>
-          <t>1. Attempt the gated action directly via the API (bypassing the UI), e.g. completing without the required invoice.
-2. Observe whether the backend rejects (403/422) or allows it (200/201).</t>
+          <t>1. Attempt a setting-violating action directly via the API (bypassing the UI), e.g. completing without the required invoice, and note the response.
+2. As a role that lacks the mapped atom, attempt the gated action via the API and note the response.
+3. As a role that has only Work Orders: Create &amp; Edit, attempt to receive onto a work order and note the response.</t>
         </is>
       </c>
       <c r="J137" s="21" t="inlineStr">
         <is>
-          <t>1. PENDING DECISION: determine whether the backend enforces the setting (rejects) or the gate is front-end only (allows).</t>
+          <t>1. The backend enforces the Simple-Flow settings and the permission atoms (it is not front-end only): a setting-violating or unauthorized request is rejected.
+2. Because several work-order atoms collapse to the same backend role pair, any role with Work Orders: Create &amp; Edit can receive onto a work order.
+3. The receive endpoint accepts the documented OR of ROLE_DELIVERY_CREATE_AND_EDIT, ROLE_WORK_ORDER_PART_CREATE and ROLE_WORK_ORDER_CREATE_AND_EDIT.</t>
         </is>
       </c>
       <c r="K137" s="21" t="inlineStr">
         <is>
-          <t>requirements §8 open questions</t>
-        </is>
-      </c>
-      <c r="L137" s="18" t="inlineStr">
-        <is>
-          <t>Open-Question</t>
+          <t>requirements §9.4 (BE enforcement + atom collapse)</t>
+        </is>
+      </c>
+      <c r="L137" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="M137" s="21" t="inlineStr">
         <is>
-          <t>§8 asks whether BE should enforce Simple-Flow settings. Hypothesis from Custom Roles: BE often enforces only resource-level View/Edit while granular gates are FE-only. Verify; do not assume. See Open Questions.</t>
+          <t>Answered by SV-8183: BE DOES enforce the Simple-Flow settings and atoms (change from the Custom Roles FE-only finding), subject to the WO-atom collapse caveat (SV-7864). Not yet driven live.</t>
         </is>
       </c>
     </row>
@@ -10778,7 +10802,7 @@
       </c>
       <c r="D138" s="17" t="inlineStr">
         <is>
-          <t>Verify whether review role-gating uses custom roles or is open for v1</t>
+          <t>Verify review sign-off is governed by the Review Work Orders custom-role permission (not open to all)</t>
         </is>
       </c>
       <c r="E138" s="25" t="inlineStr">
@@ -10793,1373 +10817,1590 @@
       </c>
       <c r="G138" s="17" t="inlineStr">
         <is>
-          <t>Depends on permissions matrix (TBD).</t>
+          <t>Review Work Orders permission + reviewer must not be the completer.</t>
         </is>
       </c>
       <c r="H138" s="17" t="inlineStr">
         <is>
-          <t>1. Credentials for several roles exist.
-2. A work order in Review state exists.</t>
+          <t>1. Credentials for roles with and without Review Work Orders exist.
+2. A work order in Review state exists, sent to review by a known user.</t>
         </is>
       </c>
       <c r="I138" s="17" t="inlineStr">
         <is>
-          <t>1. Determine which roles can sign off review.
-2. Determine whether this is governed by a custom-role permission or open to all.</t>
+          <t>1. Confirm that only roles holding Review Work Orders can sign off, and roles without it cannot.
+2. Confirm the user who completed / sent the work order to review cannot sign it off.</t>
         </is>
       </c>
       <c r="J138" s="17" t="inlineStr">
         <is>
-          <t>1. PENDING DECISION: whether review sign-off is gated by custom roles or open for v1 is unresolved.</t>
+          <t>1. Review sign-off is governed by the Review Work Orders custom-role permission (it is NOT open to all users for v1).
+2. The permission gates the Mark Reviewed action, and the reviewer-not-completer rule is enforced (the completer cannot sign off).</t>
         </is>
       </c>
       <c r="K138" s="17" t="inlineStr">
         <is>
-          <t>requirements §8 open questions</t>
-        </is>
-      </c>
-      <c r="L138" s="18" t="inlineStr">
-        <is>
-          <t>Open-Question</t>
+          <t>requirements R7 / §9 (Review Work Orders + reviewer != completer)</t>
+        </is>
+      </c>
+      <c r="L138" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="M138" s="17" t="inlineStr">
         <is>
-          <t>Explicit open question. See Open Questions.</t>
+          <t>Answered by SV-8183: review sign-off = Review Work Orders atom (custom-role gated, not open for v1) plus the reviewer != completer NET-NEW rule. Role-gating negatives not yet verified live.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="20" t="inlineStr">
         <is>
+          <t>SF-PERM-08</t>
+        </is>
+      </c>
+      <c r="B139" s="21" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C139" s="21" t="inlineStr">
+        <is>
+          <t>R7 (reviewer != completer)</t>
+        </is>
+      </c>
+      <c r="D139" s="21" t="inlineStr">
+        <is>
+          <t>Verify the user who completed or sent the work order to review cannot Mark Reviewed it</t>
+        </is>
+      </c>
+      <c r="E139" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F139" s="21" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="G139" s="21" t="inlineStr">
+        <is>
+          <t>Review Work Orders permission + reviewer must not be the completer.</t>
+        </is>
+      </c>
+      <c r="H139" s="21" t="inlineStr">
+        <is>
+          <t>1. Two different users who both hold the Review Work Orders permission exist.
+2. User A has completed / sent a work order to review; it is in Review state.</t>
+        </is>
+      </c>
+      <c r="I139" s="21" t="inlineStr">
+        <is>
+          <t>1. Sign in as User A (who sent the work order to review) and open the work order in Review.
+2. Attempt to Mark Reviewed.
+3. Sign in as User B (a different user who holds Review Work Orders) and Mark Reviewed.</t>
+        </is>
+      </c>
+      <c r="J139" s="21" t="inlineStr">
+        <is>
+          <t>1. User A cannot Mark Reviewed the work order they completed / sent to review; the action is blocked or disabled.
+2. User B, a different user who holds the Review Work Orders permission, can Mark Reviewed and sign off.
+3. The reviewer must be a different person from the completer.</t>
+        </is>
+      </c>
+      <c r="K139" s="21" t="inlineStr">
+        <is>
+          <t>requirements R7 / §9 (reviewer != completer NET-NEW rule)</t>
+        </is>
+      </c>
+      <c r="L139" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M139" s="21" t="inlineStr">
+        <is>
+          <t>NET-NEW hard rule from SV-8183: stamp sentToReviewBy/completedBy and block Mark Reviewed for that user. Role-gating negatives not yet verified live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="16" t="inlineStr">
+        <is>
+          <t>SF-PERM-09</t>
+        </is>
+      </c>
+      <c r="B140" s="17" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C140" s="17" t="inlineStr">
+        <is>
+          <t>S5 / §9 (See Financial Data gate)</t>
+        </is>
+      </c>
+      <c r="D140" s="17" t="inlineStr">
+        <is>
+          <t>Verify a Technician cannot add a vendorless / no-part-number part (lacks See Financial Data)</t>
+        </is>
+      </c>
+      <c r="E140" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F140" s="17" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="G140" s="17" t="inlineStr">
+        <is>
+          <t>WO Lines: Create &amp; Edit + See Financial Data. Technician has WO Lines: Create &amp; Edit but no See Financial Data.</t>
+        </is>
+      </c>
+      <c r="H140" s="17" t="inlineStr">
+        <is>
+          <t>1. A Technician credential exists (WO Lines: Create &amp; Edit, no See Financial Data).
+2. An open work order with a line is available.</t>
+        </is>
+      </c>
+      <c r="I140" s="17" t="inlineStr">
+        <is>
+          <t>1. Sign in as the Technician and open the work order line.
+2. Attempt to add a vendorless / no-part-number part (description + quantity + sell price).</t>
+        </is>
+      </c>
+      <c r="J140" s="17" t="inlineStr">
+        <is>
+          <t>1. The Technician cannot add a vendorless / no-part-number part.
+2. The mandatory sell price cannot be entered without See Financial Data, so the add is prevented.</t>
+        </is>
+      </c>
+      <c r="K140" s="17" t="inlineStr">
+        <is>
+          <t>requirements S5 / §9 (Decision 4)</t>
+        </is>
+      </c>
+      <c r="L140" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M140" s="17" t="inlineStr">
+        <is>
+          <t>SV-8183 Decision 4: adding a vendorless part requires See Financial Data (sell is mandatory, no catalog source). Role-gating negative not yet verified live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="20" t="inlineStr">
+        <is>
+          <t>SF-PERM-10</t>
+        </is>
+      </c>
+      <c r="B141" s="21" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C141" s="21" t="inlineStr">
+        <is>
+          <t>§9 per-role completion matrix</t>
+        </is>
+      </c>
+      <c r="D141" s="21" t="inlineStr">
+        <is>
+          <t>Verify the Complete Work Order action follows the per-role completion permission matrix</t>
+        </is>
+      </c>
+      <c r="E141" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F141" s="21" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="G141" s="21" t="inlineStr">
+        <is>
+          <t>Work Orders: Create &amp; Edit + WO Lines: Create &amp; Edit + Full View.</t>
+        </is>
+      </c>
+      <c r="H141" s="21" t="inlineStr">
+        <is>
+          <t>1. Credentials for each system role exist (Admin, Service Manager, Senior SA, Service Advisor, Foreman, Technician, Parts Manager, Parts Tech, Office, Sales Rep, Time Clock).
+2. A work order ready to complete is available.</t>
+        </is>
+      </c>
+      <c r="I141" s="21" t="inlineStr">
+        <is>
+          <t>1. For each role, open the work order and check whether the Complete Work Order action is available and usable.
+2. Record the result per role against the checklist below.
+3. Roles expected to be able to complete: Admin, Service Manager, Senior SA, Service Advisor, Foreman, Parts Manager.
+4. Roles expected NOT to be able to complete: Technician, Parts Tech, Office, Sales Rep, Time Clock.</t>
+        </is>
+      </c>
+      <c r="J141" s="21" t="inlineStr">
+        <is>
+          <t>1. Complete Work Order is available for Admin, Service Manager, Senior SA, Service Advisor, Foreman and Parts Manager.
+2. Complete Work Order is NOT available for Technician, Parts Tech, Office, Sales Rep or Time Clock.
+3. Technician and Parts Tech are blocked because they cannot approve lines and/or lack Work Orders: Create &amp; Edit; Office is view-only; Sales Rep and Time Clock have no work-order edit access.</t>
+        </is>
+      </c>
+      <c r="K141" s="21" t="inlineStr">
+        <is>
+          <t>requirements §9 (per-role matrix)</t>
+        </is>
+      </c>
+      <c r="L141" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M141" s="21" t="inlineStr">
+        <is>
+          <t>Per-role completion checklist derived from the SV-8183 role matrix. Role-gating negatives not yet verified live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="16" t="inlineStr">
+        <is>
           <t>SF-VAL-01</t>
         </is>
       </c>
-      <c r="B139" s="21" t="inlineStr">
+      <c r="B142" s="17" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C139" s="21" t="inlineStr">
+      <c r="C142" s="17" t="inlineStr">
         <is>
           <t>S2-R2 / S3-R3 / S4-R3</t>
         </is>
       </c>
-      <c r="D139" s="21" t="inlineStr">
+      <c r="D142" s="17" t="inlineStr">
         <is>
           <t>Verify completion is blocked when required mileage is missing</t>
         </is>
       </c>
-      <c r="E139" s="22" t="inlineStr">
+      <c r="E142" s="22" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F139" s="21" t="inlineStr">
+      <c r="F142" s="17" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G139" s="21" t="inlineStr">
+      <c r="G142" s="17" t="inlineStr">
         <is>
           <t>Work Order edit access.</t>
         </is>
       </c>
-      <c r="H139" s="21" t="inlineStr">
+      <c r="H142" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. Require Mileage is ON and the work order has no mileage.</t>
         </is>
       </c>
-      <c r="I139" s="21" t="inlineStr">
+      <c r="I142" s="17" t="inlineStr">
         <is>
           <t>1. Start completion.
 2. Leave mileage empty and try to proceed.</t>
         </is>
       </c>
-      <c r="J139" s="21" t="inlineStr">
+      <c r="J142" s="17" t="inlineStr">
         <is>
           <t>1. Completion is blocked until mileage is entered.</t>
         </is>
       </c>
-      <c r="K139" s="21" t="inlineStr">
+      <c r="K142" s="17" t="inlineStr">
         <is>
           <t>WO Review Flow.html (Details step)</t>
         </is>
       </c>
-      <c r="L139" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M139" s="21" t="inlineStr">
+      <c r="L142" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M142" s="17" t="inlineStr">
         <is>
           <t>Details step seen (S2-13) but empty-field block not isolated. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" s="16" t="inlineStr">
+    <row r="143">
+      <c r="A143" s="20" t="inlineStr">
         <is>
           <t>SF-VAL-02</t>
         </is>
       </c>
-      <c r="B140" s="17" t="inlineStr">
+      <c r="B143" s="21" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C140" s="17" t="inlineStr">
+      <c r="C143" s="21" t="inlineStr">
         <is>
           <t>S15-R2 / S3-R3</t>
         </is>
       </c>
-      <c r="D140" s="17" t="inlineStr">
+      <c r="D143" s="21" t="inlineStr">
         <is>
           <t>Verify completion is blocked when a required VIN is missing (non-review flow)</t>
         </is>
       </c>
-      <c r="E140" s="23" t="inlineStr">
+      <c r="E143" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F140" s="17" t="inlineStr">
+      <c r="F143" s="21" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G140" s="17" t="inlineStr">
+      <c r="G143" s="21" t="inlineStr">
         <is>
           <t>Work Order edit access.</t>
         </is>
       </c>
-      <c r="H140" s="17" t="inlineStr">
+      <c r="H143" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. VIN is required for this org's completion and the work order has no VIN.
 3. Require Review is OFF (VIN is collected at completion in the non-review flow).</t>
         </is>
       </c>
-      <c r="I140" s="17" t="inlineStr">
+      <c r="I143" s="21" t="inlineStr">
         <is>
           <t>1. Start completion.
 2. Leave VIN empty and try to proceed.</t>
         </is>
       </c>
-      <c r="J140" s="17" t="inlineStr">
+      <c r="J143" s="21" t="inlineStr">
         <is>
           <t>1. Completion is blocked until the VIN is entered.</t>
         </is>
       </c>
-      <c r="K140" s="17" t="inlineStr">
+      <c r="K143" s="21" t="inlineStr">
         <is>
           <t>requirements S15-R2</t>
         </is>
       </c>
-      <c r="L140" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M140" s="17" t="inlineStr">
+      <c r="L143" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M143" s="21" t="inlineStr">
         <is>
           <t>Not isolated in VIU. Needs live verification. (In review flow, VIN is captured at Mark Reviewed — see SF-REV-06.)</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="20" t="inlineStr">
+    <row r="144">
+      <c r="A144" s="16" t="inlineStr">
         <is>
           <t>SF-VAL-03</t>
         </is>
       </c>
-      <c r="B141" s="21" t="inlineStr">
+      <c r="B144" s="17" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C141" s="21" t="inlineStr">
+      <c r="C144" s="17" t="inlineStr">
         <is>
           <t>S3-R3 / S4-R3</t>
         </is>
       </c>
-      <c r="D141" s="21" t="inlineStr">
+      <c r="D144" s="17" t="inlineStr">
         <is>
           <t>Verify completion is blocked when required engine hours are missing</t>
         </is>
       </c>
-      <c r="E141" s="23" t="inlineStr">
+      <c r="E144" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F141" s="21" t="inlineStr">
+      <c r="F144" s="17" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G141" s="21" t="inlineStr">
+      <c r="G144" s="17" t="inlineStr">
         <is>
           <t>Work Order edit access.</t>
         </is>
       </c>
-      <c r="H141" s="21" t="inlineStr">
+      <c r="H144" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. Require Engine Hours is ON and the work order has no engine hours.</t>
         </is>
       </c>
-      <c r="I141" s="21" t="inlineStr">
+      <c r="I144" s="17" t="inlineStr">
         <is>
           <t>1. Start completion.
 2. Leave engine hours empty and try to proceed.</t>
         </is>
       </c>
-      <c r="J141" s="21" t="inlineStr">
+      <c r="J144" s="17" t="inlineStr">
         <is>
           <t>1. Completion is blocked until engine hours are entered.</t>
         </is>
       </c>
-      <c r="K141" s="21" t="inlineStr">
+      <c r="K144" s="17" t="inlineStr">
         <is>
           <t>requirements S3-R3 / S4-R3</t>
         </is>
       </c>
-      <c r="L141" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M141" s="21" t="inlineStr">
+      <c r="L144" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M144" s="17" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="16" t="inlineStr">
+    <row r="145">
+      <c r="A145" s="20" t="inlineStr">
         <is>
           <t>SF-VAL-04</t>
         </is>
       </c>
-      <c r="B142" s="17" t="inlineStr">
+      <c r="B145" s="21" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C142" s="17" t="inlineStr">
+      <c r="C145" s="21" t="inlineStr">
         <is>
           <t>TS-R4</t>
         </is>
       </c>
-      <c r="D142" s="17" t="inlineStr">
+      <c r="D145" s="21" t="inlineStr">
         <is>
           <t>Verify the tech-story Next/Continue button stays disabled while the story textarea is empty</t>
         </is>
       </c>
-      <c r="E142" s="23" t="inlineStr">
+      <c r="E145" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F142" s="17" t="inlineStr">
+      <c r="F145" s="21" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G142" s="17" t="inlineStr">
+      <c r="G145" s="21" t="inlineStr">
         <is>
           <t>Work Order edit access.</t>
         </is>
       </c>
-      <c r="H142" s="17" t="inlineStr">
+      <c r="H145" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. The tech-story modal is open on a line.</t>
         </is>
       </c>
-      <c r="I142" s="17" t="inlineStr">
+      <c r="I145" s="21" t="inlineStr">
         <is>
           <t>1. Leave the story textarea empty.
 2. Check the Next/Continue button.
 3. Type any text and check again.</t>
         </is>
       </c>
-      <c r="J142" s="17" t="inlineStr">
+      <c r="J145" s="21" t="inlineStr">
         <is>
           <t>1. With the textarea empty, Next/Continue is disabled.
 2. After typing text, Next/Continue becomes enabled.</t>
         </is>
       </c>
-      <c r="K142" s="17" t="inlineStr">
+      <c r="K145" s="21" t="inlineStr">
         <is>
           <t>WO Review Flow.html</t>
         </is>
       </c>
-      <c r="L142" s="19" t="inlineStr">
+      <c r="L145" s="19" t="inlineStr">
         <is>
           <t>VIU-Verified</t>
         </is>
       </c>
-      <c r="M142" s="17" t="inlineStr">
+      <c r="M145" s="21" t="inlineStr">
         <is>
           <t>Verified 2026-07-06 — Continue disabled until non-empty (S2-11-techstory.png).</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="20" t="inlineStr">
+    <row r="146">
+      <c r="A146" s="16" t="inlineStr">
         <is>
           <t>SF-VAL-05</t>
         </is>
       </c>
-      <c r="B143" s="21" t="inlineStr">
+      <c r="B146" s="17" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C143" s="21" t="inlineStr">
+      <c r="C146" s="17" t="inlineStr">
         <is>
           <t>S3-R3 / S4-R5 / §4</t>
         </is>
       </c>
-      <c r="D143" s="21" t="inlineStr">
+      <c r="D146" s="17" t="inlineStr">
         <is>
           <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
         </is>
       </c>
-      <c r="E143" s="22" t="inlineStr">
+      <c r="E146" s="22" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F143" s="21" t="inlineStr">
+      <c r="F146" s="17" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G143" s="21" t="inlineStr">
+      <c r="G146" s="17" t="inlineStr">
         <is>
           <t>receive access.</t>
         </is>
       </c>
-      <c r="H143" s="21" t="inlineStr">
+      <c r="H146" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. Require Vendor Invoice Number is ON and a part is being received.</t>
         </is>
       </c>
-      <c r="I143" s="21" t="inlineStr">
+      <c r="I146" s="17" t="inlineStr">
         <is>
           <t>1. On the receive surface, leave the vendor invoice number empty.
 2. Attempt to receive.</t>
         </is>
       </c>
-      <c r="J143" s="21" t="inlineStr">
+      <c r="J146" s="17" t="inlineStr">
         <is>
           <t>1. Receiving is blocked without a vendor invoice number.
 2. Once an invoice number is entered, receiving is allowed.</t>
         </is>
       </c>
-      <c r="K143" s="21" t="inlineStr">
+      <c r="K146" s="17" t="inlineStr">
         <is>
           <t>requirements §4 / S4-R5</t>
         </is>
       </c>
-      <c r="L143" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M143" s="21" t="inlineStr">
+      <c r="L146" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M146" s="17" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="16" t="inlineStr">
+    <row r="147">
+      <c r="A147" s="20" t="inlineStr">
         <is>
           <t>SF-VAL-06</t>
         </is>
       </c>
-      <c r="B144" s="17" t="inlineStr">
+      <c r="B147" s="21" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C144" s="17" t="inlineStr">
+      <c r="C147" s="21" t="inlineStr">
         <is>
           <t>S10 / S12-R2 / S13</t>
         </is>
       </c>
-      <c r="D144" s="17" t="inlineStr">
+      <c r="D147" s="21" t="inlineStr">
         <is>
           <t>Verify a vendor-missing part cannot be received without both a vendor and a part number</t>
         </is>
       </c>
-      <c r="E144" s="22" t="inlineStr">
+      <c r="E147" s="22" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F144" s="17" t="inlineStr">
+      <c r="F147" s="21" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G144" s="17" t="inlineStr">
+      <c r="G147" s="21" t="inlineStr">
         <is>
           <t>receive access.</t>
         </is>
       </c>
-      <c r="H144" s="17" t="inlineStr">
+      <c r="H147" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A vendor-missing part is on a receive surface.</t>
         </is>
       </c>
-      <c r="I144" s="17" t="inlineStr">
+      <c r="I147" s="21" t="inlineStr">
         <is>
           <t>1. Attempt to receive with no vendor.
 2. Attempt to receive with a vendor but no part number.
 3. Provide both and receive.</t>
         </is>
       </c>
-      <c r="J144" s="17" t="inlineStr">
+      <c r="J147" s="21" t="inlineStr">
         <is>
           <t>1. Receiving is blocked without a vendor.
 2. Receiving is blocked without a part number.
 3. Receiving succeeds only with both.</t>
         </is>
       </c>
-      <c r="K144" s="17" t="inlineStr">
+      <c r="K147" s="21" t="inlineStr">
         <is>
           <t>requirements S12-R2 / S10</t>
         </is>
       </c>
-      <c r="L144" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M144" s="17" t="inlineStr">
+      <c r="L147" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M147" s="21" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="20" t="inlineStr">
+    <row r="148">
+      <c r="A148" s="16" t="inlineStr">
         <is>
           <t>SF-VAL-07</t>
         </is>
       </c>
-      <c r="B145" s="21" t="inlineStr">
+      <c r="B148" s="17" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C145" s="21" t="inlineStr">
+      <c r="C148" s="17" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
-      <c r="D145" s="21" t="inlineStr">
+      <c r="D148" s="17" t="inlineStr">
         <is>
           <t>Verify Confirm Review is disabled until a VIN is entered in the Mark Reviewed dialog</t>
         </is>
       </c>
-      <c r="E145" s="23" t="inlineStr">
+      <c r="E148" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F145" s="21" t="inlineStr">
+      <c r="F148" s="17" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G145" s="21" t="inlineStr">
+      <c r="G148" s="17" t="inlineStr">
         <is>
           <t>Reviewer role (matrix TBD).</t>
         </is>
       </c>
-      <c r="H145" s="21" t="inlineStr">
+      <c r="H148" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. The Mark Reviewed dialog is open on a WO with no VIN on the asset.</t>
         </is>
       </c>
-      <c r="I145" s="21" t="inlineStr">
+      <c r="I148" s="17" t="inlineStr">
         <is>
           <t>1. Clear the VIN field.
 2. Check the Confirm Review button.
 3. Enter a VIN and check again.</t>
         </is>
       </c>
-      <c r="J145" s="21" t="inlineStr">
+      <c r="J148" s="17" t="inlineStr">
         <is>
           <t>1. Confirm Review is disabled while VIN is empty.
 2. Confirm Review enables after a VIN is entered.</t>
         </is>
       </c>
-      <c r="K145" s="21" t="inlineStr">
+      <c r="K148" s="17" t="inlineStr">
         <is>
           <t>WO Review Flow.html; requirements R7</t>
         </is>
       </c>
-      <c r="L145" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M145" s="21" t="inlineStr">
+      <c r="L148" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M148" s="17" t="inlineStr">
         <is>
           <t>In VIU the VIN was pre-filled from the asset, so the empty-VIN disabled state was not forced. Needs a WO with no VIN to verify.</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="16" t="inlineStr">
+    <row r="149">
+      <c r="A149" s="20" t="inlineStr">
         <is>
           <t>SF-VAL-08</t>
         </is>
       </c>
-      <c r="B146" s="17" t="inlineStr">
+      <c r="B149" s="21" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C146" s="17" t="inlineStr">
+      <c r="C149" s="21" t="inlineStr">
         <is>
           <t>S3-R9 (idempotency)</t>
         </is>
       </c>
-      <c r="D146" s="17" t="inlineStr">
+      <c r="D149" s="21" t="inlineStr">
         <is>
           <t>Verify re-completing after cancelling does not create duplicate POs</t>
         </is>
       </c>
-      <c r="E146" s="23" t="inlineStr">
+      <c r="E149" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F146" s="17" t="inlineStr">
+      <c r="F149" s="21" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G146" s="17" t="inlineStr">
+      <c r="G149" s="21" t="inlineStr">
         <is>
           <t>Work Order edit access.</t>
         </is>
       </c>
-      <c r="H146" s="17" t="inlineStr">
+      <c r="H149" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A part-bearing work order had completion started and cancelled once.</t>
         </is>
       </c>
-      <c r="I146" s="17" t="inlineStr">
+      <c r="I149" s="21" t="inlineStr">
         <is>
           <t>1. Cancel the first completion attempt.
 2. Start and complete again.
 3. Inspect the POs.</t>
         </is>
       </c>
-      <c r="J146" s="17" t="inlineStr">
+      <c r="J149" s="21" t="inlineStr">
         <is>
           <t>1. No duplicate POs are created on the second attempt.</t>
         </is>
       </c>
-      <c r="K146" s="17" t="inlineStr">
+      <c r="K149" s="21" t="inlineStr">
         <is>
           <t>requirements S3-R9</t>
         </is>
       </c>
-      <c r="L146" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M146" s="17" t="inlineStr">
+      <c r="L149" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M149" s="21" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification. (Also covered from the flow side in SF-COMP-23.)</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="20" t="inlineStr">
+    <row r="150">
+      <c r="A150" s="16" t="inlineStr">
         <is>
           <t>SF-VAL-09</t>
         </is>
       </c>
-      <c r="B147" s="21" t="inlineStr">
+      <c r="B150" s="17" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C147" s="21" t="inlineStr">
+      <c r="C150" s="17" t="inlineStr">
         <is>
           <t>S8-R7 / §4 field locking</t>
         </is>
       </c>
-      <c r="D147" s="21" t="inlineStr">
+      <c r="D150" s="17" t="inlineStr">
         <is>
           <t>Verify the sell field is locked after the work order is invoiced/paid with a lock icon and tooltip</t>
         </is>
       </c>
-      <c r="E147" s="23" t="inlineStr">
+      <c r="E150" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F147" s="21" t="inlineStr">
+      <c r="F150" s="17" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G147" s="21" t="inlineStr">
+      <c r="G150" s="17" t="inlineStr">
         <is>
           <t>receive access.</t>
         </is>
       </c>
-      <c r="H147" s="21" t="inlineStr">
+      <c r="H150" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A part on an invoiced/paid work order is on a receive surface.</t>
         </is>
       </c>
-      <c r="I147" s="21" t="inlineStr">
+      <c r="I150" s="17" t="inlineStr">
         <is>
           <t>1. Open the receive surface for the invoiced/paid WO part.
 2. Try to edit the sell field.
 3. Hover the lock icon.</t>
         </is>
       </c>
-      <c r="J147" s="21" t="inlineStr">
+      <c r="J150" s="17" t="inlineStr">
         <is>
           <t>1. The sell field is locked (not editable).
 2. A lock icon and tooltip 'Locked — this part is already invoiced or paid' are shown.
 3. Only cost remains editable.</t>
         </is>
       </c>
-      <c r="K147" s="21" t="inlineStr">
+      <c r="K150" s="17" t="inlineStr">
         <is>
           <t>requirements S8-R7 / §4</t>
         </is>
       </c>
-      <c r="L147" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M147" s="21" t="inlineStr">
+      <c r="L150" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M150" s="17" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="16" t="inlineStr">
+    <row r="151">
+      <c r="A151" s="20" t="inlineStr">
         <is>
           <t>SF-VAL-10</t>
         </is>
       </c>
-      <c r="B148" s="17" t="inlineStr">
+      <c r="B151" s="21" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C148" s="17" t="inlineStr">
+      <c r="C151" s="21" t="inlineStr">
         <is>
           <t>S9-R3 / §4 (uniqueness relaxed)</t>
         </is>
       </c>
-      <c r="D148" s="17" t="inlineStr">
+      <c r="D151" s="21" t="inlineStr">
         <is>
           <t>Verify the same vendor invoice number can be reused across POs (uniqueness relaxed)</t>
         </is>
       </c>
-      <c r="E148" s="25" t="inlineStr">
+      <c r="E151" s="25" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F148" s="17" t="inlineStr">
+      <c r="F151" s="21" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G148" s="17" t="inlineStr">
+      <c r="G151" s="21" t="inlineStr">
         <is>
           <t>receive access.</t>
         </is>
       </c>
-      <c r="H148" s="17" t="inlineStr">
+      <c r="H151" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. Two POs for the same vendor are being received.</t>
         </is>
       </c>
-      <c r="I148" s="17" t="inlineStr">
+      <c r="I151" s="21" t="inlineStr">
         <is>
           <t>1. Enter the same invoice number on both POs.
 2. Receive both.</t>
         </is>
       </c>
-      <c r="J148" s="17" t="inlineStr">
+      <c r="J151" s="21" t="inlineStr">
         <is>
           <t>1. The reused invoice number is accepted (uniqueness is relaxed).
 2. Both POs receive successfully.</t>
         </is>
       </c>
-      <c r="K148" s="17" t="inlineStr">
+      <c r="K151" s="21" t="inlineStr">
         <is>
           <t>requirements S9-R3 / §4</t>
         </is>
       </c>
-      <c r="L148" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M148" s="17" t="inlineStr">
+      <c r="L151" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M151" s="21" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="20" t="inlineStr">
+    <row r="152">
+      <c r="A152" s="16" t="inlineStr">
         <is>
           <t>SF-VAL-11</t>
         </is>
       </c>
-      <c r="B149" s="21" t="inlineStr">
+      <c r="B152" s="17" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C149" s="21" t="inlineStr">
+      <c r="C152" s="17" t="inlineStr">
         <is>
           <t>Key Decision (line approval)</t>
         </is>
       </c>
-      <c r="D149" s="21" t="inlineStr">
+      <c r="D152" s="17" t="inlineStr">
         <is>
           <t>Verify the approve-line error text appears when completing with an unapproved line</t>
         </is>
       </c>
-      <c r="E149" s="23" t="inlineStr">
+      <c r="E152" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F149" s="21" t="inlineStr">
+      <c r="F152" s="17" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="G149" s="21" t="inlineStr">
+      <c r="G152" s="17" t="inlineStr">
         <is>
           <t>Work Order edit access.</t>
         </is>
       </c>
-      <c r="H149" s="21" t="inlineStr">
+      <c r="H152" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A work order has one unapproved line and all other gates satisfied.</t>
         </is>
       </c>
-      <c r="I149" s="21" t="inlineStr">
+      <c r="I152" s="17" t="inlineStr">
         <is>
           <t>1. Click Complete Work Order.
 2. Read the error shown at the final confirm.</t>
         </is>
       </c>
-      <c r="J149" s="21" t="inlineStr">
+      <c r="J152" s="17" t="inlineStr">
         <is>
           <t>1. The existing 'you need to approve the line to complete the work order' error is shown.
 2. Completion does not proceed until the line is approved.</t>
         </is>
       </c>
-      <c r="K149" s="21" t="inlineStr">
+      <c r="K152" s="17" t="inlineStr">
         <is>
           <t>requirements §4 Key Decision</t>
         </is>
       </c>
-      <c r="L149" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M149" s="21" t="inlineStr">
+      <c r="L152" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M152" s="17" t="inlineStr">
         <is>
           <t>PARTIAL in VIU — error not cleanly isolated (S17-02-approval-error.png). Needs a WO whose only blocker is the unapproved line.</t>
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="16" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="20" t="inlineStr">
         <is>
           <t>SF-QB-01</t>
         </is>
       </c>
-      <c r="B150" s="17" t="inlineStr">
+      <c r="B153" s="21" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C150" s="17" t="inlineStr">
+      <c r="C153" s="21" t="inlineStr">
         <is>
           <t>§5 invariant 1</t>
         </is>
       </c>
-      <c r="D150" s="17" t="inlineStr">
+      <c r="D153" s="21" t="inlineStr">
         <is>
           <t>Verify in-stock parts decrement inventory and write Part History on simple completion (skip path still runs lifecycle)</t>
         </is>
       </c>
-      <c r="E150" s="22" t="inlineStr">
+      <c r="E153" s="22" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F150" s="17" t="inlineStr">
+      <c r="F153" s="21" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G150" s="17" t="inlineStr">
+      <c r="G153" s="21" t="inlineStr">
         <is>
           <t>Work Order edit access + Inventory visibility.</t>
         </is>
       </c>
-      <c r="H150" s="17" t="inlineStr">
+      <c r="H153" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A work order has an in-stock inventory part; its on-hand quantity is noted.</t>
         </is>
       </c>
-      <c r="I150" s="17" t="inlineStr">
+      <c r="I153" s="21" t="inlineStr">
         <is>
           <t>1. Complete the work order via the simple (skip) path.
 2. Check the part's on-hand quantity and Part History.</t>
         </is>
       </c>
-      <c r="J150" s="17" t="inlineStr">
+      <c r="J153" s="21" t="inlineStr">
         <is>
           <t>1. The in-stock part's on-hand quantity decrements.
 2. A Part History entry is written.
 3. The skip path's status setter does not bypass inventory movement / Part History / catalog / delivery.</t>
         </is>
       </c>
-      <c r="K150" s="17" t="inlineStr">
+      <c r="K153" s="21" t="inlineStr">
         <is>
           <t>requirements §5 invariant 1</t>
         </is>
       </c>
-      <c r="L150" s="18" t="inlineStr">
+      <c r="L153" s="18" t="inlineStr">
         <is>
           <t>Open-Question</t>
         </is>
       </c>
-      <c r="M150" s="17" t="inlineStr">
+      <c r="M153" s="21" t="inlineStr">
         <is>
           <t>§8 open question: auto-receive of in-stock inventory on simple completion is unconfirmed, and the spec flags the bare status setter as an integrity risk. Not driven in VIU. See Open Questions.</t>
         </is>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="20" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="16" t="inlineStr">
         <is>
           <t>SF-QB-02</t>
         </is>
       </c>
-      <c r="B151" s="21" t="inlineStr">
+      <c r="B154" s="17" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C151" s="21" t="inlineStr">
+      <c r="C154" s="17" t="inlineStr">
         <is>
           <t>§5 / §4 (Create POs OFF)</t>
         </is>
       </c>
-      <c r="D151" s="21" t="inlineStr">
+      <c r="D154" s="17" t="inlineStr">
         <is>
           <t>Verify Create POs OFF produces no PO, vendor bill or AP sync and no catalog/inventory sync</t>
         </is>
       </c>
-      <c r="E151" s="22" t="inlineStr">
+      <c r="E154" s="22" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F151" s="21" t="inlineStr">
+      <c r="F154" s="17" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G151" s="21" t="inlineStr">
+      <c r="G154" s="17" t="inlineStr">
         <is>
           <t>Admin / owner (settings) + Work Order edit access + QuickBooks visibility.</t>
         </is>
       </c>
-      <c r="H151" s="21" t="inlineStr">
+      <c r="H154" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. Create Purchase Orders is OFF (see SF-SET-03).
 3. A work order with a vendor/found part exists.</t>
         </is>
       </c>
-      <c r="I151" s="21" t="inlineStr">
+      <c r="I154" s="17" t="inlineStr">
         <is>
           <t>1. Complete the work order with Create POs OFF.
 2. Check for any PO, vendor bill, AP sync.
 3. Check for any catalog/inventory sync of the vendor/found part.</t>
         </is>
       </c>
-      <c r="J151" s="21" t="inlineStr">
+      <c r="J154" s="17" t="inlineStr">
         <is>
           <t>1. EXPECTED PER SPEC: no PO, no vendor bill, no AP sync.
 2. No catalog/inventory sync (part is received at request time only).</t>
         </is>
       </c>
-      <c r="K151" s="21" t="inlineStr">
+      <c r="K154" s="17" t="inlineStr">
         <is>
           <t>requirements §4 / §5</t>
         </is>
       </c>
-      <c r="L151" s="18" t="inlineStr">
+      <c r="L154" s="18" t="inlineStr">
         <is>
           <t>Open-Question</t>
         </is>
       </c>
-      <c r="M151" s="21" t="inlineStr">
+      <c r="M154" s="17" t="inlineStr">
         <is>
           <t>Blocked by VIU bug #1: no 'Create Purchase Orders' toggle exists, so Create POs OFF cannot be configured. See Open Questions.</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="16" t="inlineStr">
+    <row r="155">
+      <c r="A155" s="20" t="inlineStr">
         <is>
           <t>SF-QB-03</t>
         </is>
       </c>
-      <c r="B152" s="17" t="inlineStr">
+      <c r="B155" s="21" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C152" s="17" t="inlineStr">
+      <c r="C155" s="21" t="inlineStr">
         <is>
           <t>§5 invariant 2</t>
         </is>
       </c>
-      <c r="D152" s="17" t="inlineStr">
+      <c r="D155" s="21" t="inlineStr">
         <is>
           <t>Verify POs ON plus receiving runs the full pipeline: receive → Delivery → Vendor Bill → QuickBooks (both surfaces sync)</t>
         </is>
       </c>
-      <c r="E152" s="22" t="inlineStr">
+      <c r="E155" s="22" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F152" s="17" t="inlineStr">
+      <c r="F155" s="21" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G152" s="17" t="inlineStr">
+      <c r="G155" s="21" t="inlineStr">
         <is>
           <t>receive access + QuickBooks visibility.</t>
         </is>
       </c>
-      <c r="H152" s="17" t="inlineStr">
+      <c r="H155" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. Create POs is on and a work order has a receivable vendor part.</t>
         </is>
       </c>
-      <c r="I152" s="17" t="inlineStr">
+      <c r="I155" s="21" t="inlineStr">
         <is>
           <t>1. Receive the part via Accept Delivery.
 2. Check that a Delivery, then a Vendor Bill, then a QuickBooks sync occur.
 3. Repeat via the Bulk Receive surface (once built) and confirm it also syncs.</t>
         </is>
       </c>
-      <c r="J152" s="17" t="inlineStr">
+      <c r="J155" s="21" t="inlineStr">
         <is>
           <t>1. Receiving creates a Delivery, then a Vendor Bill, then syncs to QuickBooks.
 2. Both receive surfaces sync the vendor bill (only complete-simple bypasses this).</t>
         </is>
       </c>
-      <c r="K152" s="17" t="inlineStr">
+      <c r="K155" s="21" t="inlineStr">
         <is>
           <t>requirements §5 invariant 2</t>
         </is>
       </c>
-      <c r="L152" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M152" s="17" t="inlineStr">
+      <c r="L155" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M155" s="21" t="inlineStr">
         <is>
           <t>Not driven in VIU; needs QuickBooks inspection. Bulk Receive surface not yet built. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="20" t="inlineStr">
+    <row r="156">
+      <c r="A156" s="16" t="inlineStr">
         <is>
           <t>SF-QB-04</t>
         </is>
       </c>
-      <c r="B153" s="21" t="inlineStr">
+      <c r="B156" s="17" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C153" s="21" t="inlineStr">
+      <c r="C156" s="17" t="inlineStr">
         <is>
           <t>§5 (vendorless/no-PN)</t>
         </is>
       </c>
-      <c r="D153" s="21" t="inlineStr">
+      <c r="D156" s="17" t="inlineStr">
         <is>
           <t>Verify a vendorless / no-PN part has zero inventory interaction until a vendor and/or part number is added</t>
         </is>
       </c>
-      <c r="E153" s="23" t="inlineStr">
+      <c r="E156" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F153" s="21" t="inlineStr">
+      <c r="F156" s="17" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G153" s="21" t="inlineStr">
+      <c r="G156" s="17" t="inlineStr">
         <is>
           <t>Inventory visibility.</t>
         </is>
       </c>
-      <c r="H153" s="21" t="inlineStr">
+      <c r="H156" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A vendorless / no-PN part exists on a work order.</t>
         </is>
       </c>
-      <c r="I153" s="21" t="inlineStr">
+      <c r="I156" s="17" t="inlineStr">
         <is>
           <t>1. Before adding a vendor/PN, check inventory and Part History for the part.
 2. Add a vendor and PN, then re-check.</t>
         </is>
       </c>
-      <c r="J153" s="21" t="inlineStr">
+      <c r="J156" s="17" t="inlineStr">
         <is>
           <t>1. Before a vendor/PN, there is zero inventory interaction (no item, no history).
 2. After a vendor and PN are added, normal inventory handling applies.</t>
         </is>
       </c>
-      <c r="K153" s="21" t="inlineStr">
+      <c r="K156" s="17" t="inlineStr">
         <is>
           <t>requirements §5</t>
         </is>
       </c>
-      <c r="L153" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M153" s="21" t="inlineStr">
+      <c r="L156" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M156" s="17" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="16" t="inlineStr">
+    <row r="157">
+      <c r="A157" s="20" t="inlineStr">
         <is>
           <t>SF-QB-05</t>
         </is>
       </c>
-      <c r="B154" s="17" t="inlineStr">
+      <c r="B157" s="21" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C154" s="17" t="inlineStr">
+      <c r="C157" s="21" t="inlineStr">
         <is>
           <t>§5 / S6-R3</t>
         </is>
       </c>
-      <c r="D154" s="17" t="inlineStr">
+      <c r="D157" s="21" t="inlineStr">
         <is>
           <t>Verify Vendor Missing POs are excluded from QuickBooks until a vendor and part number are provided</t>
         </is>
       </c>
-      <c r="E154" s="23" t="inlineStr">
+      <c r="E157" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F154" s="17" t="inlineStr">
+      <c r="F157" s="21" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G154" s="17" t="inlineStr">
+      <c r="G157" s="21" t="inlineStr">
         <is>
           <t>QuickBooks visibility.</t>
         </is>
       </c>
-      <c r="H154" s="17" t="inlineStr">
+      <c r="H157" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A Vendor Missing PO exists.</t>
         </is>
       </c>
-      <c r="I154" s="17" t="inlineStr">
+      <c r="I157" s="21" t="inlineStr">
         <is>
           <t>1. Check QuickBooks sync for the Vendor Missing PO.
 2. Provide a vendor and part number and re-check.</t>
         </is>
       </c>
-      <c r="J154" s="17" t="inlineStr">
+      <c r="J157" s="21" t="inlineStr">
         <is>
           <t>1. While vendor/PN are missing, the PO is excluded from QuickBooks.
 2. Once both are provided, it becomes eligible for QuickBooks.</t>
         </is>
       </c>
-      <c r="K154" s="17" t="inlineStr">
+      <c r="K157" s="21" t="inlineStr">
         <is>
           <t>requirements §5 / S6-R3</t>
         </is>
       </c>
-      <c r="L154" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M154" s="17" t="inlineStr">
+      <c r="L157" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M157" s="21" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="20" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="16" t="inlineStr">
         <is>
           <t>SF-QB-06</t>
         </is>
       </c>
-      <c r="B155" s="21" t="inlineStr">
+      <c r="B158" s="17" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C155" s="21" t="inlineStr">
+      <c r="C158" s="17" t="inlineStr">
         <is>
           <t>§8 (cost at completion)</t>
         </is>
       </c>
-      <c r="D155" s="21" t="inlineStr">
+      <c r="D158" s="17" t="inlineStr">
         <is>
           <t>Verify cost at completion behavior to avoid $0-cost margins in QuickBooks</t>
         </is>
       </c>
-      <c r="E155" s="23" t="inlineStr">
+      <c r="E158" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F155" s="21" t="inlineStr">
+      <c r="F158" s="17" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G155" s="21" t="inlineStr">
-        <is>
-          <t>Work Order edit access + QuickBooks visibility.</t>
-        </is>
-      </c>
-      <c r="H155" s="21" t="inlineStr">
+      <c r="G158" s="17" t="inlineStr">
+        <is>
+          <t>Work Order edit access + See Financial Data + QuickBooks visibility.</t>
+        </is>
+      </c>
+      <c r="H158" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A work order has a part with no cost recorded at completion.</t>
         </is>
       </c>
-      <c r="I155" s="21" t="inlineStr">
+      <c r="I158" s="17" t="inlineStr">
         <is>
           <t>1. Complete the work order.
 2. Check the resulting cost/margin figures that flow to QuickBooks.</t>
         </is>
       </c>
-      <c r="J155" s="21" t="inlineStr">
-        <is>
-          <t>1. PENDING DECISION: whether cost can be entered at completion to avoid $0-cost margins is unresolved. Confirm the intended behavior.</t>
-        </is>
-      </c>
-      <c r="K155" s="21" t="inlineStr">
-        <is>
-          <t>requirements §8 open questions</t>
-        </is>
-      </c>
-      <c r="L155" s="18" t="inlineStr">
-        <is>
-          <t>Open-Question</t>
-        </is>
-      </c>
-      <c r="M155" s="21" t="inlineStr">
-        <is>
-          <t>§8 open question. Not driven in VIU. See Open Questions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="16" t="inlineStr">
+      <c r="J158" s="17" t="inlineStr">
+        <is>
+          <t>1. The cost and margin values sent to QuickBooks at completion are recorded and checked for any $0-cost margins.
+2. For vendorless / no-part-number parts the mandatory sell price is captured at add time behind the See Financial Data gate, so a completing user has a sell figure and $0-cost margins are avoided.</t>
+        </is>
+      </c>
+      <c r="K158" s="17" t="inlineStr">
+        <is>
+          <t>requirements §9 (See Financial Data gate on vendorless sell)</t>
+        </is>
+      </c>
+      <c r="L158" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M158" s="17" t="inlineStr">
+        <is>
+          <t>Resolved by SV-8183 (Decision 4): the cost-at-completion concern is addressed by requiring See Financial Data to enter the mandatory sell on a vendorless add. Money figures still need live verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="20" t="inlineStr">
         <is>
           <t>SF-QB-07</t>
         </is>
       </c>
-      <c r="B156" s="17" t="inlineStr">
+      <c r="B159" s="21" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C156" s="17" t="inlineStr">
+      <c r="C159" s="21" t="inlineStr">
         <is>
           <t>§5 (Journal Entry / Inventory → QBO)</t>
         </is>
       </c>
-      <c r="D156" s="17" t="inlineStr">
+      <c r="D159" s="21" t="inlineStr">
         <is>
           <t>Verify the Journal Entry / Inventory sync to QuickBooks fires on invoice creation (not PO-dependent)</t>
         </is>
       </c>
-      <c r="E156" s="23" t="inlineStr">
+      <c r="E159" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F156" s="17" t="inlineStr">
+      <c r="F159" s="21" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G156" s="17" t="inlineStr">
+      <c r="G159" s="21" t="inlineStr">
         <is>
           <t>Finance access + QuickBooks visibility.</t>
         </is>
       </c>
-      <c r="H156" s="17" t="inlineStr">
+      <c r="H159" s="21" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A completed work order is ready to invoice.</t>
         </is>
       </c>
-      <c r="I156" s="17" t="inlineStr">
+      <c r="I159" s="21" t="inlineStr">
         <is>
           <t>1. Create the invoice.
 2. Check for the Journal Entry / Inventory sync to QuickBooks.</t>
         </is>
       </c>
-      <c r="J156" s="17" t="inlineStr">
+      <c r="J159" s="21" t="inlineStr">
         <is>
           <t>1. The Journal Entry / Inventory sync to QuickBooks fires on invoice creation.
 2. This sync is not dependent on a PO existing.</t>
         </is>
       </c>
-      <c r="K156" s="17" t="inlineStr">
+      <c r="K159" s="21" t="inlineStr">
         <is>
           <t>requirements §5</t>
         </is>
       </c>
-      <c r="L156" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M156" s="17" t="inlineStr">
+      <c r="L159" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M159" s="21" t="inlineStr">
         <is>
           <t>Not driven in VIU; needs QuickBooks inspection. Needs live verification.</t>
         </is>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="20" t="inlineStr">
+    <row r="160">
+      <c r="A160" s="16" t="inlineStr">
         <is>
           <t>SF-QB-08</t>
         </is>
       </c>
-      <c r="B157" s="21" t="inlineStr">
+      <c r="B160" s="17" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C157" s="21" t="inlineStr">
+      <c r="C160" s="17" t="inlineStr">
         <is>
           <t>§5 invariant 3</t>
         </is>
       </c>
-      <c r="D157" s="21" t="inlineStr">
+      <c r="D160" s="17" t="inlineStr">
         <is>
           <t>Verify Inventory Part History is preserved for any part that becomes inventory-tracked</t>
         </is>
       </c>
-      <c r="E157" s="23" t="inlineStr">
+      <c r="E160" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F157" s="21" t="inlineStr">
+      <c r="F160" s="17" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="G157" s="21" t="inlineStr">
+      <c r="G160" s="17" t="inlineStr">
         <is>
           <t>Inventory visibility.</t>
         </is>
       </c>
-      <c r="H157" s="21" t="inlineStr">
+      <c r="H160" s="17" t="inlineStr">
         <is>
           <t>1. Signed in as Admin.
 2. A part transitions to inventory-tracked (e.g. a part number is added and it is received).</t>
         </is>
       </c>
-      <c r="I157" s="21" t="inlineStr">
+      <c r="I160" s="17" t="inlineStr">
         <is>
           <t>1. Add a part number to a previously untracked part and receive it.
 2. Open the item's Part History.</t>
         </is>
       </c>
-      <c r="J157" s="21" t="inlineStr">
+      <c r="J160" s="17" t="inlineStr">
         <is>
           <t>1. Part History is preserved / created for the now inventory-tracked part.</t>
         </is>
       </c>
-      <c r="K157" s="21" t="inlineStr">
+      <c r="K160" s="17" t="inlineStr">
         <is>
           <t>requirements §5 invariant 3</t>
         </is>
       </c>
-      <c r="L157" s="24" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="M157" s="21" t="inlineStr">
+      <c r="L160" s="24" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="M160" s="17" t="inlineStr">
         <is>
           <t>Not driven in VIU. Needs live verification.</t>
         </is>
@@ -12176,7 +12417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14710,7 +14951,7 @@
       </c>
       <c r="C88" s="21" t="inlineStr">
         <is>
-          <t>Verify Mark Reviewed is available only to manager/foreman and disabled for an advisor with 'Awaiting review'</t>
+          <t>Verify Mark Reviewed is gated by the Review Work Orders permission and disabled for a role without it</t>
         </is>
       </c>
       <c r="D88" s="21" t="inlineStr">
@@ -14874,7 +15115,7 @@
     <row r="94">
       <c r="A94" s="20" t="inlineStr">
         <is>
-          <t>SF-PERM-05</t>
+          <t>SF-PERM-02</t>
         </is>
       </c>
       <c r="B94" s="21" t="inlineStr">
@@ -14884,7 +15125,7 @@
       </c>
       <c r="C94" s="21" t="inlineStr">
         <is>
-          <t>Verify the PO Receive button is hidden for office/readonly users</t>
+          <t>Verify which roles can complete a work order (Simple completion)</t>
         </is>
       </c>
       <c r="D94" s="21" t="inlineStr">
@@ -14903,17 +15144,17 @@
     <row r="95">
       <c r="A95" s="16" t="inlineStr">
         <is>
-          <t>SF-VAL-01</t>
+          <t>SF-PERM-03</t>
         </is>
       </c>
       <c r="B95" s="17" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C95" s="17" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when required mileage is missing</t>
+          <t>Verify which roles can perform Bulk Receive</t>
         </is>
       </c>
       <c r="D95" s="17" t="inlineStr">
@@ -14923,7 +15164,7 @@
       </c>
       <c r="E95" s="17" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F95" s="17" t="inlineStr"/>
@@ -14932,17 +15173,17 @@
     <row r="96">
       <c r="A96" s="20" t="inlineStr">
         <is>
-          <t>SF-VAL-02</t>
+          <t>SF-PERM-04</t>
         </is>
       </c>
       <c r="B96" s="21" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C96" s="21" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when a required VIN is missing (non-review flow)</t>
+          <t>Verify which roles can Mark Reviewed (sign off)</t>
         </is>
       </c>
       <c r="D96" s="21" t="inlineStr">
@@ -14952,7 +15193,7 @@
       </c>
       <c r="E96" s="21" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F96" s="21" t="inlineStr"/>
@@ -14961,17 +15202,17 @@
     <row r="97">
       <c r="A97" s="16" t="inlineStr">
         <is>
-          <t>SF-VAL-03</t>
+          <t>SF-PERM-05</t>
         </is>
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when required engine hours are missing</t>
+          <t>Verify the PO Receive button is hidden for office/readonly users</t>
         </is>
       </c>
       <c r="D97" s="17" t="inlineStr">
@@ -14981,7 +15222,7 @@
       </c>
       <c r="E97" s="17" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F97" s="17" t="inlineStr"/>
@@ -14990,17 +15231,17 @@
     <row r="98">
       <c r="A98" s="20" t="inlineStr">
         <is>
-          <t>SF-VAL-05</t>
+          <t>SF-PERM-06</t>
         </is>
       </c>
       <c r="B98" s="21" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C98" s="21" t="inlineStr">
         <is>
-          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
+          <t>Verify the backend enforces the Simple-Flow settings and permission atoms (not front-end only)</t>
         </is>
       </c>
       <c r="D98" s="21" t="inlineStr">
@@ -15010,7 +15251,7 @@
       </c>
       <c r="E98" s="21" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F98" s="21" t="inlineStr"/>
@@ -15019,17 +15260,17 @@
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
         <is>
-          <t>SF-VAL-06</t>
+          <t>SF-PERM-07</t>
         </is>
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
         <is>
-          <t>Verify a vendor-missing part cannot be received without both a vendor and a part number</t>
+          <t>Verify review sign-off is governed by the Review Work Orders custom-role permission (not open to all)</t>
         </is>
       </c>
       <c r="D99" s="17" t="inlineStr">
@@ -15039,7 +15280,7 @@
       </c>
       <c r="E99" s="17" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F99" s="17" t="inlineStr"/>
@@ -15048,17 +15289,17 @@
     <row r="100">
       <c r="A100" s="20" t="inlineStr">
         <is>
-          <t>SF-VAL-07</t>
+          <t>SF-PERM-08</t>
         </is>
       </c>
       <c r="B100" s="21" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C100" s="21" t="inlineStr">
         <is>
-          <t>Verify Confirm Review is disabled until a VIN is entered in the Mark Reviewed dialog</t>
+          <t>Verify the user who completed or sent the work order to review cannot Mark Reviewed it</t>
         </is>
       </c>
       <c r="D100" s="21" t="inlineStr">
@@ -15068,7 +15309,7 @@
       </c>
       <c r="E100" s="21" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F100" s="21" t="inlineStr"/>
@@ -15077,17 +15318,17 @@
     <row r="101">
       <c r="A101" s="16" t="inlineStr">
         <is>
-          <t>SF-VAL-08</t>
+          <t>SF-PERM-09</t>
         </is>
       </c>
       <c r="B101" s="17" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
         <is>
-          <t>Verify re-completing after cancelling does not create duplicate POs</t>
+          <t>Verify a Technician cannot add a vendorless / no-part-number part (lacks See Financial Data)</t>
         </is>
       </c>
       <c r="D101" s="17" t="inlineStr">
@@ -15097,7 +15338,7 @@
       </c>
       <c r="E101" s="17" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F101" s="17" t="inlineStr"/>
@@ -15106,17 +15347,17 @@
     <row r="102">
       <c r="A102" s="20" t="inlineStr">
         <is>
-          <t>SF-VAL-09</t>
+          <t>SF-PERM-10</t>
         </is>
       </c>
       <c r="B102" s="21" t="inlineStr">
         <is>
-          <t>Validation / Edge</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="C102" s="21" t="inlineStr">
         <is>
-          <t>Verify the sell field is locked after the work order is invoiced/paid with a lock icon and tooltip</t>
+          <t>Verify the Complete Work Order action follows the per-role completion permission matrix</t>
         </is>
       </c>
       <c r="D102" s="21" t="inlineStr">
@@ -15126,7 +15367,7 @@
       </c>
       <c r="E102" s="21" t="inlineStr">
         <is>
-          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+          <t>Role/cookie-dependent - needs a non-admin (or manager/foreman/office) credential; only the admin session works on sv7301 (tech key = 403). Expected also depends on the permissions matrix (TBD).</t>
         </is>
       </c>
       <c r="F102" s="21" t="inlineStr"/>
@@ -15135,7 +15376,7 @@
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
         <is>
-          <t>SF-VAL-10</t>
+          <t>SF-VAL-01</t>
         </is>
       </c>
       <c r="B103" s="17" t="inlineStr">
@@ -15145,7 +15386,7 @@
       </c>
       <c r="C103" s="17" t="inlineStr">
         <is>
-          <t>Verify the same vendor invoice number can be reused across POs (uniqueness relaxed)</t>
+          <t>Verify completion is blocked when required mileage is missing</t>
         </is>
       </c>
       <c r="D103" s="17" t="inlineStr">
@@ -15164,7 +15405,7 @@
     <row r="104">
       <c r="A104" s="20" t="inlineStr">
         <is>
-          <t>SF-VAL-11</t>
+          <t>SF-VAL-02</t>
         </is>
       </c>
       <c r="B104" s="21" t="inlineStr">
@@ -15174,7 +15415,7 @@
       </c>
       <c r="C104" s="21" t="inlineStr">
         <is>
-          <t>Verify the approve-line error text appears when completing with an unapproved line</t>
+          <t>Verify completion is blocked when a required VIN is missing (non-review flow)</t>
         </is>
       </c>
       <c r="D104" s="21" t="inlineStr">
@@ -15193,17 +15434,17 @@
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
         <is>
-          <t>SF-QB-03</t>
+          <t>SF-VAL-03</t>
         </is>
       </c>
       <c r="B105" s="17" t="inlineStr">
         <is>
-          <t>QuickBooks / Inventory Integrity</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
         <is>
-          <t>Verify POs ON plus receiving runs the full pipeline: receive → Delivery → Vendor Bill → QuickBooks (both surfaces sync)</t>
+          <t>Verify completion is blocked when required engine hours are missing</t>
         </is>
       </c>
       <c r="D105" s="17" t="inlineStr">
@@ -15213,7 +15454,7 @@
       </c>
       <c r="E105" s="17" t="inlineStr">
         <is>
-          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
         </is>
       </c>
       <c r="F105" s="17" t="inlineStr"/>
@@ -15222,17 +15463,17 @@
     <row r="106">
       <c r="A106" s="20" t="inlineStr">
         <is>
-          <t>SF-QB-04</t>
+          <t>SF-VAL-05</t>
         </is>
       </c>
       <c r="B106" s="21" t="inlineStr">
         <is>
-          <t>QuickBooks / Inventory Integrity</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C106" s="21" t="inlineStr">
         <is>
-          <t>Verify a vendorless / no-PN part has zero inventory interaction until a vendor and/or part number is added</t>
+          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
         </is>
       </c>
       <c r="D106" s="21" t="inlineStr">
@@ -15242,7 +15483,7 @@
       </c>
       <c r="E106" s="21" t="inlineStr">
         <is>
-          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
         </is>
       </c>
       <c r="F106" s="21" t="inlineStr"/>
@@ -15251,17 +15492,17 @@
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
         <is>
-          <t>SF-QB-05</t>
+          <t>SF-VAL-06</t>
         </is>
       </c>
       <c r="B107" s="17" t="inlineStr">
         <is>
-          <t>QuickBooks / Inventory Integrity</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
         <is>
-          <t>Verify Vendor Missing POs are excluded from QuickBooks until a vendor and part number are provided</t>
+          <t>Verify a vendor-missing part cannot be received without both a vendor and a part number</t>
         </is>
       </c>
       <c r="D107" s="17" t="inlineStr">
@@ -15271,7 +15512,7 @@
       </c>
       <c r="E107" s="17" t="inlineStr">
         <is>
-          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
         </is>
       </c>
       <c r="F107" s="17" t="inlineStr"/>
@@ -15280,17 +15521,17 @@
     <row r="108">
       <c r="A108" s="20" t="inlineStr">
         <is>
-          <t>SF-QB-07</t>
+          <t>SF-VAL-07</t>
         </is>
       </c>
       <c r="B108" s="21" t="inlineStr">
         <is>
-          <t>QuickBooks / Inventory Integrity</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C108" s="21" t="inlineStr">
         <is>
-          <t>Verify the Journal Entry / Inventory sync to QuickBooks fires on invoice creation (not PO-dependent)</t>
+          <t>Verify Confirm Review is disabled until a VIN is entered in the Mark Reviewed dialog</t>
         </is>
       </c>
       <c r="D108" s="21" t="inlineStr">
@@ -15300,7 +15541,7 @@
       </c>
       <c r="E108" s="21" t="inlineStr">
         <is>
-          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
         </is>
       </c>
       <c r="F108" s="21" t="inlineStr"/>
@@ -15309,17 +15550,17 @@
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
         <is>
-          <t>SF-QB-08</t>
+          <t>SF-VAL-08</t>
         </is>
       </c>
       <c r="B109" s="17" t="inlineStr">
         <is>
-          <t>QuickBooks / Inventory Integrity</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>Verify Inventory Part History is preserved for any part that becomes inventory-tracked</t>
+          <t>Verify re-completing after cancelling does not create duplicate POs</t>
         </is>
       </c>
       <c r="D109" s="17" t="inlineStr">
@@ -15329,11 +15570,272 @@
       </c>
       <c r="E109" s="17" t="inlineStr">
         <is>
-          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
         </is>
       </c>
       <c r="F109" s="17" t="inlineStr"/>
       <c r="G109" s="17" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="20" t="inlineStr">
+        <is>
+          <t>SF-VAL-09</t>
+        </is>
+      </c>
+      <c r="B110" s="21" t="inlineStr">
+        <is>
+          <t>Validation / Edge</t>
+        </is>
+      </c>
+      <c r="C110" s="21" t="inlineStr">
+        <is>
+          <t>Verify the sell field is locked after the work order is invoiced/paid with a lock icon and tooltip</t>
+        </is>
+      </c>
+      <c r="D110" s="21" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E110" s="21" t="inlineStr">
+        <is>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+        </is>
+      </c>
+      <c r="F110" s="21" t="inlineStr"/>
+      <c r="G110" s="21" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
+        <is>
+          <t>SF-VAL-10</t>
+        </is>
+      </c>
+      <c r="B111" s="17" t="inlineStr">
+        <is>
+          <t>Validation / Edge</t>
+        </is>
+      </c>
+      <c r="C111" s="17" t="inlineStr">
+        <is>
+          <t>Verify the same vendor invoice number can be reused across POs (uniqueness relaxed)</t>
+        </is>
+      </c>
+      <c r="D111" s="17" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E111" s="17" t="inlineStr">
+        <is>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+        </is>
+      </c>
+      <c r="F111" s="17" t="inlineStr"/>
+      <c r="G111" s="17" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="20" t="inlineStr">
+        <is>
+          <t>SF-VAL-11</t>
+        </is>
+      </c>
+      <c r="B112" s="21" t="inlineStr">
+        <is>
+          <t>Validation / Edge</t>
+        </is>
+      </c>
+      <c r="C112" s="21" t="inlineStr">
+        <is>
+          <t>Verify the approve-line error text appears when completing with an unapproved line</t>
+        </is>
+      </c>
+      <c r="D112" s="21" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E112" s="21" t="inlineStr">
+        <is>
+          <t>Not driven in the VIU run - needs a targeted live walk on sv7301.</t>
+        </is>
+      </c>
+      <c r="F112" s="21" t="inlineStr"/>
+      <c r="G112" s="21" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="16" t="inlineStr">
+        <is>
+          <t>SF-QB-03</t>
+        </is>
+      </c>
+      <c r="B113" s="17" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="C113" s="17" t="inlineStr">
+        <is>
+          <t>Verify POs ON plus receiving runs the full pipeline: receive → Delivery → Vendor Bill → QuickBooks (both surfaces sync)</t>
+        </is>
+      </c>
+      <c r="D113" s="17" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E113" s="17" t="inlineStr">
+        <is>
+          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+        </is>
+      </c>
+      <c r="F113" s="17" t="inlineStr"/>
+      <c r="G113" s="17" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="20" t="inlineStr">
+        <is>
+          <t>SF-QB-04</t>
+        </is>
+      </c>
+      <c r="B114" s="21" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="C114" s="21" t="inlineStr">
+        <is>
+          <t>Verify a vendorless / no-PN part has zero inventory interaction until a vendor and/or part number is added</t>
+        </is>
+      </c>
+      <c r="D114" s="21" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E114" s="21" t="inlineStr">
+        <is>
+          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+        </is>
+      </c>
+      <c r="F114" s="21" t="inlineStr"/>
+      <c r="G114" s="21" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="16" t="inlineStr">
+        <is>
+          <t>SF-QB-05</t>
+        </is>
+      </c>
+      <c r="B115" s="17" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="C115" s="17" t="inlineStr">
+        <is>
+          <t>Verify Vendor Missing POs are excluded from QuickBooks until a vendor and part number are provided</t>
+        </is>
+      </c>
+      <c r="D115" s="17" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E115" s="17" t="inlineStr">
+        <is>
+          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+        </is>
+      </c>
+      <c r="F115" s="17" t="inlineStr"/>
+      <c r="G115" s="17" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="20" t="inlineStr">
+        <is>
+          <t>SF-QB-06</t>
+        </is>
+      </c>
+      <c r="B116" s="21" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="C116" s="21" t="inlineStr">
+        <is>
+          <t>Verify cost at completion behavior to avoid $0-cost margins in QuickBooks</t>
+        </is>
+      </c>
+      <c r="D116" s="21" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E116" s="21" t="inlineStr">
+        <is>
+          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+        </is>
+      </c>
+      <c r="F116" s="21" t="inlineStr"/>
+      <c r="G116" s="21" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="16" t="inlineStr">
+        <is>
+          <t>SF-QB-07</t>
+        </is>
+      </c>
+      <c r="B117" s="17" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="C117" s="17" t="inlineStr">
+        <is>
+          <t>Verify the Journal Entry / Inventory sync to QuickBooks fires on invoice creation (not PO-dependent)</t>
+        </is>
+      </c>
+      <c r="D117" s="17" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E117" s="17" t="inlineStr">
+        <is>
+          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+        </is>
+      </c>
+      <c r="F117" s="17" t="inlineStr"/>
+      <c r="G117" s="17" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="20" t="inlineStr">
+        <is>
+          <t>SF-QB-08</t>
+        </is>
+      </c>
+      <c r="B118" s="21" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="C118" s="21" t="inlineStr">
+        <is>
+          <t>Verify Inventory Part History is preserved for any part that becomes inventory-tracked</t>
+        </is>
+      </c>
+      <c r="D118" s="21" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E118" s="21" t="inlineStr">
+        <is>
+          <t>Needs QuickBooks / inventory inspection after a live receive/invoice.</t>
+        </is>
+      </c>
+      <c r="F118" s="21" t="inlineStr"/>
+      <c r="G118" s="21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -15349,14 +15851,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15385,6 +15888,11 @@
           <t>Affected cases</t>
         </is>
       </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Status / Resolution</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="27" t="n">
@@ -15397,22 +15905,27 @@
       </c>
       <c r="C2" s="21" t="inlineStr">
         <is>
-          <t>The spec supplies NO consolidated permissions/role matrix (§8 flags it as unresolved). Which roles may complete WOs, bulk receive, edit settings, and sign off review is undefined. Role-gating cases are authored but their expected results are TBD.</t>
+          <t>The spec supplied NO consolidated permissions/role matrix (§8 flagged it as unresolved). Which roles may complete WOs, bulk receive, edit settings, and sign off review was undefined.</t>
         </is>
       </c>
       <c r="D2" s="21" t="inlineStr">
         <is>
-          <t>Every role-gating case's expected result is a guess without this. Hypothesis to verify (from Custom Roles): the backend may enforce only resource-level View/Edit while granular gates are front-end display only.</t>
+          <t>Every role-gating case's expected result depended on this.</t>
         </is>
       </c>
       <c r="E2" s="21" t="inlineStr">
         <is>
-          <t>SF-PERM-01..07, SF-SET-11, SF-RCV-03, SF-REV-09</t>
+          <t>SF-PERM-01..10, SF-SET-11, SF-RCV-03, SF-REV-09</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>RESOLVED by SV-8183. Simple Flow adds NO new permission atom - every action maps to an existing Custom Roles atom (see requirements §9 action-&gt;atom map + per-role matrix): Settings = App Settings (defaults Admin/Service Manager/Office); Complete WO = Work Orders C&amp;E + WO Lines C&amp;E/Full View; Bulk Receive = Vendor &amp; Order Mgmt C&amp;E + See Financial Data; Receive-on-WO = Order Parts (FE); Mark Reviewed = Review Work Orders + reviewer != completer. Source: SV-8183.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="n">
+      <c r="A3" s="29" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="17" t="inlineStr">
@@ -15433,6 +15946,11 @@
       <c r="E3" s="17" t="inlineStr">
         <is>
           <t>Global - especially SF-SET-08, SF-TECH-08, SF-REV-08</t>
+        </is>
+      </c>
+      <c r="F3" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
         </is>
       </c>
     </row>
@@ -15460,14 +15978,19 @@
           <t>SF-SET-08</t>
         </is>
       </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Explicitly NOT addressed by SV-8183.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="n">
+      <c r="A5" s="29" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>'Create Purchase Orders' toggle absent (VIU bug #1)</t>
+          <t>'Create Purchase Orders' toggle absent (build deviation #1)</t>
         </is>
       </c>
       <c r="C5" s="17" t="inlineStr">
@@ -15483,6 +16006,11 @@
       <c r="E5" s="17" t="inlineStr">
         <is>
           <t>SF-SET-03, SF-COMP-06, SF-QB-02</t>
+        </is>
+      </c>
+      <c r="F5" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Explicitly NOT addressed by SV-8183.</t>
         </is>
       </c>
     </row>
@@ -15502,7 +16030,7 @@
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Determines whether the tech-story gate-modal cases are authoritative. VIU showed the gate-modal working, so Story 17 appears current - confirm.</t>
+          <t>Determines whether the tech-story gate-modal cases are authoritative. The live build showed the gate-modal working, so Story 17 appears current - confirm.</t>
         </is>
       </c>
       <c r="E6" s="21" t="inlineStr">
@@ -15510,9 +16038,14 @@
           <t>SF-TECH-08 (and all SF-TECH-*)</t>
         </is>
       </c>
+      <c r="F6" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="n">
+      <c r="A7" s="29" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="17" t="inlineStr">
@@ -15533,6 +16066,11 @@
       <c r="E7" s="17" t="inlineStr">
         <is>
           <t>SF-QB-06</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>RESOLVED by SV-8183 (Decision 4). A vendorless / no-PN part add requires See Financial Data, so the mandatory sell price is captured at add time and $0-cost margins are avoided. Source: SV-8183.</t>
         </is>
       </c>
     </row>
@@ -15560,9 +16098,14 @@
           <t>SF-COMP-07, SF-QB-01</t>
         </is>
       </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="n">
+      <c r="A9" s="29" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="17" t="inlineStr">
@@ -15577,12 +16120,17 @@
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>Sets the expected result for API-level negative tests (403/422 vs 200/201). Custom Roles precedent: BE often enforces only resource-level View/Edit.</t>
+          <t>Sets the expected result for API-level negative tests (403/422 vs 200/201).</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t>SF-PERM-06</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>RESOLVED by SV-8183. The backend DOES enforce the Simple-Flow settings AND the permission atoms (not FE-only), subject to the WO-atom collapse caveat: any role with WO Create &amp; Edit can receive onto a WO, and the receive endpoint accepts the OR of ROLE_DELIVERY_CREATE_AND_EDIT / ROLE_WORK_ORDER_PART_CREATE / ROLE_WORK_ORDER_CREATE_AND_EDIT. Source: SV-8183.</t>
         </is>
       </c>
     </row>
@@ -15592,7 +16140,7 @@
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>Save Settings always enabled (VIU bug #2)</t>
+          <t>Save Settings always enabled (build deviation #2)</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
@@ -15610,14 +16158,19 @@
           <t>SF-SET-13</t>
         </is>
       </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="n">
+      <c r="A11" s="29" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>Mark Reviewed missing optional note (VIU bug #3)</t>
+          <t>Mark Reviewed missing optional note (build deviation #3)</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
@@ -15633,6 +16186,11 @@
       <c r="E11" s="17" t="inlineStr">
         <is>
           <t>SF-REV-10</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
         </is>
       </c>
     </row>
@@ -15642,7 +16200,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Review sign-off jumps to Complete (VIU bug #4)</t>
+          <t>Review sign-off jumps to Complete (build deviation #4)</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
@@ -15660,9 +16218,14 @@
           <t>SF-REV-08, SF-REV-11</t>
         </is>
       </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="n">
+      <c r="A13" s="29" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="17" t="inlineStr">
@@ -15683,6 +16246,11 @@
       <c r="E13" s="17" t="inlineStr">
         <is>
           <t>SF-UX-04</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
         </is>
       </c>
     </row>
@@ -15710,9 +16278,14 @@
           <t>SF-REV-15</t>
         </is>
       </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. SV-8183 defined WHO can sign off review, but NOT the require-review default cohort.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="n">
+      <c r="A15" s="29" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="17" t="inlineStr">
@@ -15733,6 +16306,11 @@
       <c r="E15" s="17" t="inlineStr">
         <is>
           <t>SF-RCV-05, SF-RCV-07</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>OPEN - pending Milos. Not addressed by SV-8183.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simple Flow: finalize SV-8183 live VIU — deliverables + state, TestRail sync staged (1 update_case, not executed)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_V1_TestCases.xlsx
+++ b/build/simple-flow/SimpleFlow_V1_TestCases.xlsx
@@ -9930,7 +9930,7 @@
       </c>
       <c r="M109" s="21" t="inlineStr">
         <is>
-          <t>Reworded per Milos Round-3 split ruling (2026-07-16): Bulk Receive = top, Receive/Accept-Delivery = bottom. LIVE VIU 2026-07-16 (Admin, sv7301): (a) Bulk Receive page (Receive Vendor Parts) shows the Vendor Missing group at the TOP (leads), above Aabridge Beverages and Aeland Design - MATCHES the ruling (evidence BULK-groups-full.png). (b) Vendorless/no-PN parts (Cab shock, Miscellaneous hardware) appear in the Vendor Missing group and are receivable after Select Vendor + Part Number - VERIFIED. (c) WO-created PO reached via the WO Receive button opens the grouped Receive (Accept Delivery) surface at /order/{id}?receive=1 - VERIFIED. DEVIATION: on that Receive (Accept Delivery) screen the Vendor Missing group is currently at the TOP (leads), NOT the bottom as ruled - observed on two orders (S-15884 above Aeland Design; S-15878 above Aeboro Motors); evidence ORDER-RECV-S15884-allgroups-full.png, ORDER-RECV-S15878-full.png. Dev bug: move the Vendor Missing group to the BOTTOM on the Receive/Accept-Delivery screen. Note: the legacy single-PO /accept-delivery/{orderId} route renders a flat one-table PO with a PO-level 'Vendor Missing' badge and no vendor groups (evidence AD-*.png). || STAGING VIU 2026-07-20: Vendor Missing group + Select Vendor + Part Number entry confirmed; Bulk-Receive TOP position confirmed (matches Milos ruling). Accept-Delivery BOTTOM position not re-observed -&gt; Deviation UNCHANGED. || STAGING VIU 2026-07-20 (definitive): seeded a WO with a real-vendor group + a true vendor_id=null part, ordered into one PO, opened Accept-Delivery — Vendor Missing group renders at the TOP (y=406, before the vendor group). Milos ruled BOTTOM for that screen -&gt; DEVIATION PERSISTS. Bug draft #5 stays OPEN. Evidence: DEV-accept-delivery.png.</t>
+          <t>Reworded per Milos Round-3 split ruling (2026-07-16): Bulk Receive = top, Receive/Accept-Delivery = bottom. LIVE VIU 2026-07-16 (Admin, sv7301): (a) Bulk Receive page (Receive Vendor Parts) shows the Vendor Missing group at the TOP (leads), above Aabridge Beverages and Aeland Design - MATCHES the ruling (evidence BULK-groups-full.png). (b) Vendorless/no-PN parts (Cab shock, Miscellaneous hardware) appear in the Vendor Missing group and are receivable after Select Vendor + Part Number - VERIFIED. (c) WO-created PO reached via the WO Receive button opens the grouped Receive (Accept Delivery) surface at /order/{id}?receive=1 - VERIFIED. DEVIATION: on that Receive (Accept Delivery) screen the Vendor Missing group is currently at the TOP (leads), NOT the bottom as ruled - observed on two orders (S-15884 above Aeland Design; S-15878 above Aeboro Motors); evidence ORDER-RECV-S15884-allgroups-full.png, ORDER-RECV-S15878-full.png. Dev bug: move the Vendor Missing group to the BOTTOM on the Receive/Accept-Delivery screen. Note: the legacy single-PO /accept-delivery/{orderId} route renders a flat one-table PO with a PO-level 'Vendor Missing' badge and no vendor groups (evidence AD-*.png). || STAGING VIU 2026-07-20: Vendor Missing group + Select Vendor + Part Number entry confirmed; Bulk-Receive TOP position confirmed (matches Milos ruling). Accept-Delivery BOTTOM position not re-observed -&gt; Deviation UNCHANGED. || STAGING VIU 2026-07-20 (definitive): seeded a WO with a real-vendor group + a true vendor_id=null part, ordered into one PO, opened Accept-Delivery — Vendor Missing group renders at the TOP (y=406, before the vendor group). Milos ruled BOTTOM for that screen -&gt; DEVIATION PERSISTS. Bug draft #5 stays OPEN. Evidence: DEV-accept-delivery.png. || ACCEPTED COSMETIC DEVIATION — WON'T FIX/WON'T FILE (user decision 2026-07-20): Milos's bottom-placement ruling for the Vendor Missing group on the Accept-Delivery / 'Purchase Order Details' screen is not implemented on the build (group renders at TOP), but this is deemed PURELY VISUAL — the group still appears and functions; only its position differs. No functional/data/workflow impact. Bug draft #5 DROPPED (won't-file). viu_status stays Deviation because the build genuinely deviates from the ruling, but this is an ACCEPTED/won't-file cosmetic deviation, not an open actionable bug. No TestRail change needed — case wording already reflects the intended behavior.</t>
         </is>
       </c>
       <c r="N109" s="21" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="M111" s="21" t="inlineStr">
         <is>
-          <t>Reworded per Milos Round-3 split ruling (2026-07-16). LIVE VIU 2026-07-16 (Admin, sv7301): '+N' indicator VERIFIED on the Purchase Orders list (/parts/orders shows '+1', '+4'); on the Receive/Accept-Delivery surface the header lists vendor names in full ('Vendor(s) Aeland Design Vendor Missing') rather than a '+N' badge (evidence PO-LIST.png, ORDER-RECV-5vendor.png). Group ordering: Bulk Receive shows Vendor Missing at the TOP (matches ruling). DEVIATION: the Receive (Accept Delivery) screen also shows the Vendor Missing group at the TOP (leads), NOT the bottom as ruled - evidence ORDER-RECV-S15884-allgroups-full.png, ORDER-RECV-S15878-full.png. Same dev bug as SF-RCV-05. || STAGING VIU 2026-07-20: '+N' indicator on PO list confirmed ('+1'); Vendor Missing leads at TOP on Bulk Receive (correct per Milos). Accept-Delivery BOTTOM not re-observed -&gt; Deviation UNCHANGED. || STAGING VIU 2026-07-20 (definitive): '+N' PO-list indicator confirmed; on Accept-Delivery the Vendor Missing group is still at the TOP (should be BOTTOM per Milos) -&gt; DEVIATION PERSISTS, bug #5 stays open. Evidence: DEV-accept-delivery.png.</t>
+          <t>Reworded per Milos Round-3 split ruling (2026-07-16). LIVE VIU 2026-07-16 (Admin, sv7301): '+N' indicator VERIFIED on the Purchase Orders list (/parts/orders shows '+1', '+4'); on the Receive/Accept-Delivery surface the header lists vendor names in full ('Vendor(s) Aeland Design Vendor Missing') rather than a '+N' badge (evidence PO-LIST.png, ORDER-RECV-5vendor.png). Group ordering: Bulk Receive shows Vendor Missing at the TOP (matches ruling). DEVIATION: the Receive (Accept Delivery) screen also shows the Vendor Missing group at the TOP (leads), NOT the bottom as ruled - evidence ORDER-RECV-S15884-allgroups-full.png, ORDER-RECV-S15878-full.png. Same dev bug as SF-RCV-05. || STAGING VIU 2026-07-20: '+N' indicator on PO list confirmed ('+1'); Vendor Missing leads at TOP on Bulk Receive (correct per Milos). Accept-Delivery BOTTOM not re-observed -&gt; Deviation UNCHANGED. || STAGING VIU 2026-07-20 (definitive): '+N' PO-list indicator confirmed; on Accept-Delivery the Vendor Missing group is still at the TOP (should be BOTTOM per Milos) -&gt; DEVIATION PERSISTS, bug #5 stays open. Evidence: DEV-accept-delivery.png. || ACCEPTED COSMETIC DEVIATION — WON'T FIX/WON'T FILE (user decision 2026-07-20): Milos's bottom-placement ruling for the Vendor Missing group on the Accept-Delivery / 'Purchase Order Details' screen is not implemented on the build (group renders at TOP), but this is deemed PURELY VISUAL — the group still appears and functions; only its position differs. No functional/data/workflow impact. Bug draft #5 DROPPED (won't-file). viu_status stays Deviation because the build genuinely deviates from the ruling, but this is an ACCEPTED/won't-file cosmetic deviation, not an open actionable bug. No TestRail change needed — case wording already reflects the intended behavior.</t>
         </is>
       </c>
       <c r="N111" s="21" t="inlineStr">
@@ -13152,9 +13152,9 @@
       </c>
       <c r="J149" s="21" t="inlineStr">
         <is>
-          <t>1. Only a role with the App Settings permission (system defaults Admin, Service Manager and Office) can view and modify the Work Order settings page.
-2. A role without App Settings cannot open or change the Work Order settings.
-3. The backend rejects a Work Order settings save attempted by a role that lacks App Settings.</t>
+          <t>1. Only a role with the App Settings permission (system defaults Admin, Service Manager and Office) can open and change the Work Order settings page.
+2. A role without App Settings cannot reach the Work Order settings page (it is redirected away) and so cannot change those settings from the screen.
+3. A role that cannot open the Work Order settings page cannot save changes to it.</t>
         </is>
       </c>
       <c r="K149" s="21" t="inlineStr">

</xml_diff>